<commit_message>
Update: 2026-08-11 09:35 UTC
</commit_message>
<xml_diff>
--- a/docs/tax_updates_export.xlsx
+++ b/docs/tax_updates_export.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K39"/>
+  <dimension ref="A1:K55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -511,32 +511,32 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>VAT</t>
+          <t>Transfer Pricing</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>news</t>
+          <t>commentary</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>September 1 change: UAE announces new excise price rule for electronic smoking products - Gulf Business</t>
+          <t>Tax Insights: Canada introduces a simplified transfer pricing documentation regime - PwC</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>News — FTA Announcements</t>
+          <t>News — Big 4 UAE Tax Commentary</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -546,7 +546,7 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiwAFBVV95cUxNMXNESjR5VDVIQ0Qwb0xKUk1xRlhaTmV2RjNfdVpGaDZZYk0wcjdSbC1RRHBUNkRRaGpNOS1mSjR1blVVRHJ6MzdLeUZXM1lMWURyX21CS25DZFN3engwRWZCOFFLUDJydEEwX0pSa1lLSlNqbVlhdk9pNmtvLUh1QzFubU9RVENUNEl3QVdLc2FkRUV6TGFjZmJwLUtiUVd5dlhjVW1SLU43WFI4eGNfZkJCTXBNaEQySVR3QjZuazA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiwAFBVV95cUxOVm8yXzZQUVY4R2djbXBUdHQ0aFUyQnFaSHNxSkFCbTNxNmxSVTZVUHRxa1lvVnF2Nlk2bmhTQ2w4ejJaTVR2NUY4S3VsajBFTEV2dkRwbk9BbEh1MWtwczNVNHgtQm1yaFJwc2NlZldqM053NGhwbE1TLWR3eDNIQ3V2ZzhTQ2JmbVJlNlliMkRoalBfYzQ3WHdVaXR2R2MzNEw1dGRQNzFfRWxTWklzYkJNYVZKVjFMclFQQjIzMUU?oc=5</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr"/>
@@ -556,32 +556,32 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Corporate Tax</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>news</t>
+          <t>commentary</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>UAE small businesses claiming tax relief must still file corporate tax returns - Emirates 24|7</t>
+          <t>Canada launches public consultations on steel imports and imposes surtax on wood cabinets and vanities - EY</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>News — FTA Announcements</t>
+          <t>News — Big 4 UAE Tax Commentary</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -591,7 +591,7 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxOLXJ6YVV3T2dXazExeU04V09UYlk3NmtYT2d3Z2t1X2RPckN0RjVQZE9oNTljdi1rUUlzTDlMalotZ1JWRS03TWVFWlVVS1hyMVlDUEsxYWQ3RWgtdTdUNzVaZjE5WlhVVUhJcjkyaDFVa28yeEN2ejAtVG43dnduV2NDa0k4czRLby1sU2w2ZHZTcGtPZmpiTjRYWXB2VUExMnhreUktUDBZSkZ4LUxZYW9TYXRJc2s0U1QyMtIB1wFBVV95cUxPNWVmQzRQOEJkZnBCZVFDblE2dkFlX1hGNWlnalJBVk5QREJoU0ZvMXZIM1JJYXdLb2lQZFNnejliekY3Y29nN0tLdTUxQ0h0SUFaSVlpOWhuX3dVaHdjX3NPM1pkd2xlVDRMT1VmTHJ4QV9PbmpWRmVHRFpHZ1lyUF9ZWEJTcFJ2LS1QX0hEa0Y3dnJ4S054S211cWRMWWlHVVd2V19wQnhGa2JVR1ZxSFVNVWJMejdESlFZSkxUMGYwQUlyQkpueDlwb2dJYnlqQnZGNklscw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMigAFBVV95cUxNMy1qdEVRaXhDVUZ4c3FTNUlCS0F0SEhoRnQtRk5BTnB1d2VFSmZSUk95RmRSdEw4LUFBV1FwYTIwbTVLZHdqOEdkcDhRb29fWDc1cGN0ZFA3a0habW9iY0NWam9LZmtfa3c2NDlLZ3N1MVJYWWRwejlhM1ViSndzZg?oc=5</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr"/>
@@ -601,12 +601,12 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -621,7 +621,7 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>UAE releases registration requirements for domestic minimum top-up tax - kpmg.com</t>
+          <t>UAE extends Small Business Relief for corporate tax - Absolute Geeks</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -636,7 +636,7 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxPaGJWUy1MU0VZdmd3LTVPTmw0bDYtWlF5a3JCVkFwVnhJRUkxVkdEWUE4X1VZLXg0Tkg4YTlLWHhoOUJYVzJqR3lzUE5Pa1RpSWtjdkRDQ09UeDBoQ3Y2bGlLbkhzTXZ2WlNJeGFSLXNqRUZyRnBfNV9Mbk5UY25hdVZ6VWM2cWRYOEt4bUlnWV9QYkQtOWZudGJaV0ZJZDRVY2JGbTY1T1JTYVhyTGhEdlVuQzlzZkN6ZC1VRQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxPWU10OExoZmlXRjdCamp5VHROMnNDb1dKN1I3NE85dTI4aU84VjVvczlyanRyWEw4OVBuOWpVa1NJZm9qQ2hSZl9YYlhxOGNEYXBCeDlGQVF1RUV1TWJlSGVmdnpHRktyS2ktV2IwQ0s3T3hZMzV4Ni03aGdvVTNHZFhEYThmRE5uclJqR1BKUF90MXktS2xEaXctR0RsLXphM0g0REdvWHY?oc=5</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr"/>
@@ -646,12 +646,12 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -666,12 +666,12 @@
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>UAE Digital Economy: Why Trust, Not Speed, Now Wins The Race - Menafn</t>
+          <t>Spotify forecasts slower growth despite AI investment - Gulf Business</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>News — UAE E-Invoicing</t>
+          <t>News — FTA Announcements</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -681,7 +681,7 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMikAFBVV95cUxNbi1OcWZwSTNNYjBRZkJWS1FodlVGTG5oZHB1T3Q2cGRqazRiZGQzeUtlOVB3VXlhNUM1TnhSdW1MVS1uSng1dGFmTlAzb3ZMNXlod0c5bWo2RkdOTW1idm9JQ3dQNTM5Z3FvZl96WlNuVVh4Mmx5NGFNWXBHVFZoWnUyQU9WT01idllWclJqTXE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMilwFBVV95cUxNQUhDU0xPaGxHNTZZdDNmRFRsTndvQThIUkRVV0hyTkpVbWhFNXdsZ2hjUXFrNzByWEc1ZUdITm1FYkM2N3k5MW5paDBud1RfNGF4MXNIdlluaVktTVRfd0RlZzJpUmc0UlZ2WUlKU1VDTUdELXpoelU0Z2kteENFZjVfcWx5YmhLc21jS3J5VXVkeEZ3UXRV?oc=5</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr"/>
@@ -691,12 +691,12 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -711,12 +711,12 @@
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>Ministry of Finance sets e-cigarette liquid excise price - Sharjah24</t>
+          <t>UAE Sets Minimum Excise Price for E-Liquids - Vaping360</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>News — UAE E-Invoicing</t>
+          <t>News — FTA Announcements</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -726,7 +726,7 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiWkFVX3lxTFBGY1BCNkVheXBxM3RBdWlPNXVULWVaaWdWM3RWWU9JSWI2T3JVMGlMdl94Ync5ekFqdGU1SzAxeEMwaUhJR1hTejhVTFo4blI2Y1d5QzZUaVgwUQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMidkFVX3lxTE9HS2ZoOFFrdlRtX3N4ZXM5UlpzLTFKc21Pdi1CVkhNYW1PNGozMDBVYVZ0VjlrUDNCMFRQRG1hOGpPNllSd0dpX0dhNm02a3drdmZneHpQOUhtUkxXWlFBcDlETkt0dF9xalFRMldrVWZMSXh5NHc?oc=5</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr"/>
@@ -736,17 +736,17 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>E-Invoicing</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -756,7 +756,7 @@
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>CBUAE injects more liquidity into the banking system - EnterpriseAM</t>
+          <t>E-Invoicing Readiness Checklist: How UAE Businesses Can Prepare Before the Deadline - NewsBreak: Local News &amp; Alerts</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -771,7 +771,7 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxPRVF2amFoSUlsRENGenUxcUlxRU9NeU9QWlJhUkExb1k0cExublF1YUdrM2dJc0FySm9zQmgyQUtKU092bkpYT1I1bUhaMkxGR2o2SFVnckhIR2d4RGQzOUJnb19tZERINThyZ0NrQ1A0WUttandLcmN0QUlUaTFVZ1djMnUxdEp4SmNGMjM1Zl9HX1k?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMixgFBVV95cUxPQmFubHpKbnIzS2N1cVJkbFA5bDRWcUhzQ0lYazZ3Z0ZBazZKQzVoTjRxZXBrMFNNSGNXTGp4ZG1EZ0xTTGFwanZQZkxvbjA5UFQxYkNBLWF6bEtDSlB5UlcyNU9fc2E1VTRNMWtTYnRyOFRlTUxjRlVlcEVwRVdDb05OQlo4VC1GcUpqUkpmVzhsUmc0RGJrZlJWN0tCMXVQc0d5dTEtT055TFRDT3c5R2pUN1hpaEF3R21TOHo2d1pNZldNcUE?oc=5</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr"/>
@@ -781,12 +781,12 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -801,7 +801,7 @@
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>The Taxation Society partners with Tally Solutions to strengthen UAE's finance and tax professional community - khaleejtimes.com</t>
+          <t>A jumpy July - EnterpriseAM</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -816,7 +816,7 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi4gFBVV95cUxNMXRpRGhpQXJvUkZhQU1IcTF6Z0JtLW16cTQ1d24zZWlwQTlPMHNCeG8tY0NLc1JGcXdjT2g5V01YM3hOVmtZYzBJeThiR3hhSDRpdGdwaDhsVC1WMDFTSWN0SWdhc3hiWTRSQmV0blZEZkowYWdoSU1BaUJ6Y01ZZ2ZrWlNRc2JtUllnc0huTF92aWdmbEp4bTRvRV9fN2xTU2dmMjdLSk43ZlFlcEtuWTBKQXdFTU5pMlRnWE55VFBwcTc0STRtcFluS3Ffek1oM2NRQ1dYemVkTktESkJRSVJ30gHqAUFVX3lxTE85ZnVhMjFKMWdhenV1YlFiRGtpVTBIdjRvLVNLRFBjTHBPUnVfeG5sUGxIcWVlSlhUTEVibFV2UXdWbEg5TGNmS3hBYnczSEctV3BBT2pZT3dpcDJUeGczWE9xQ1dweV9hc1hwQnhHQkFWUDRrb0FzV0tVdmZhZ0pLZC14YlVJZjBYQmcwbUZWeG55dnhpOFliT0wxYkQ0bzl1VEhiVUpQNjQ4TVN0bFhPRERROXB5NUZZQ0VRS08tY0VmSDdLRFQzMHZ0dEZtamJ5dmp1OGZ6SmNxQjZrck8wRWs2U1A0TFJZdw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiXkFVX3lxTFBCcFdtSjE1bW5pMlREMHVqWTYwcW1xajViLWZvTmU1MUk0MUZiX2pPay12Nm5RS0tzdmJjYU9VY2hjUi10enNsYk1qcEZqc3FQc3dEZE1CaTJRYTJvVWc?oc=5</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr"/>
@@ -826,17 +826,17 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Corporate Tax</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -846,7 +846,7 @@
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>MoF extends Small Business Relief for corporate tax until end-2029 - Sharjah24</t>
+          <t>Another Hormuz workaround - EnterpriseAM</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -861,7 +861,7 @@
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiW0FVX3lxTFA4N01YTUZ2UGRGVWdDQ3JDM3JLYWJDanVuckdCLVhuQUdqUFo3clA1cGRoTUtubWNpQ0dTOUFSQk5jYzdGcVFYNkNpQjF4ckFVZ2pBc0FXM1Ffa0k?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMib0FVX3lxTE5iUjRXRTlrdVBXOHUyRWlYc2ttOXdYaVktOE5ZU1YxMnRLcnlHeWRPdl9CQmRkR3Bqc21aeFlWMmdFcGdjanc3d2RNTnRGcWdKVGdxQTZmeC02clJoSXJJaGJlUUM5TW5pQjRORkVpRQ?oc=5</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr"/>
@@ -871,17 +871,17 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>E-Invoicing</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -891,7 +891,7 @@
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>Northern Emirates’ property markets cool off + Sidara locks in USD 1.35 bn in firepower - EnterpriseAM</t>
+          <t>UAE e-invoicing: How digital invoices will transform business - Khaleej Times</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -906,7 +906,7 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxOMDUxZXd1MElSNXdaNDByLW9jbHFIenJCY21PRnhPMUx4YkdyZ1FMREVxenNWZWZUY2p3MHQ5V2xUQmswZ1RuV1g3Q3RHUzdvOFhvOGpST2diQWIwOXFBeXdzc1lYRl9FRDIxdjBjUVR3Y2VEcUdIWXB0amg4YW5qbklORzFMS3J4VUZGelkybDVZcXc0VHlNck4zTXdjR1N1UzZmSk9vSFFoMDJMVENKMFVlWEdvUTEwZFhiZmdn?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMivwFBVV95cUxQMjFwZTd6MkpqcXZKaEwxZV9fUlZWSEtSeVdIQXN6YXFPMURFMWZhOHc0NWFuWlRfd1ZNX2doQVBpbXBqRFBTOVNNcjVTYVpOcEozYmtoaWxDUHVoUFFNT1RBWEI3RzJybmFWejFNcEcxYXpybDBiUzRLUk85ajBkOHIydnBjOUV6NEVJUjZkQTNOQ0Fud1BjdGtUNVpwTmlTazdyNWZmaXRwTkthY1Nac1RPWU90T3lMemJJNHp5VdIBvwFBVV95cUxQMjFwZTd6MkpqcXZKaEwxZV9fUlZWSEtSeVdIQXN6YXFPMURFMWZhOHc0NWFuWlRfd1ZNX2doQVBpbXBqRFBTOVNNcjVTYVpOcEozYmtoaWxDUHVoUFFNT1RBWEI3RzJybmFWejFNcEcxYXpybDBiUzRLUk85ajBkOHIydnBjOUV6NEVJUjZkQTNOQ0Fud1BjdGtUNVpwTmlTazdyNWZmaXRwTkthY1Nac1RPWU90T3lMemJJNHp5VQ?oc=5</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr"/>
@@ -916,17 +916,17 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>E-Invoicing</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -936,7 +936,7 @@
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>ClearTax urges UAE businesses to prioritise execution assurance as e-invoicing decisions gather pace - Gulf News</t>
+          <t>More investments in Adnoc’s fleet, Indian IPOs, and Egypt’s North Coast - EnterpriseAM</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
@@ -951,7 +951,7 @@
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi6wFBVV95cUxPTG13TFpCRmpaaWU3ZGxsVEtqakxUUXhSc0ltWUZfOEUyWTcxWGhOZ2doazNZY1V2LWFnSlp0NHpHTXN4emN6TzFWbGlXT09xU0Q3X25BTmpBVVl0Nl9XMFdRUE9HMy1BU3BMRDFIZ1RITkw4d3BSanluZGFHal9CM3h5dDNtTlBtUG9LYXZZWkhILVZhdUpKTHhUd2lMWmVOdVJrREx4UUF4WjNvTW5hSmtBVjVyQVBpblVKa1hKbjhxRTNUVmpUMVpXOFFJSWx1NUZWUWFMYlY2ZjA2Nml6OGV6X2ZGcVhkQkQ00gH-AUFVX3lxTE12b1Q4Qjd0Rks3U1hqOC1GVTZ5RXRUOXB6eVdVd3RMTEV5Q1pRYVRrc19GaG1qY3FXRGhqMkN3N3c2emJyeTFWbEU2QkRSMHR5aWFzNlctUi1mdi1vamRHMHZoWFZlQlRCbEhrT3BLSXlsTXRfYjY4QjVHblFRU0JnZVhlam4xNEF6d0hQVUtmTHFoYnktSW5LS3dqU2VleEh4azlObnoyUTNPd2E0RWc4U0ZhMkRoc1J1c2R6VGJhc1lSYTF0cjhzdnY0Q0tvYk81YnY5UE5CdnBXZTVNQXE4UlZwMkFjbUREaEtRNlF2MWJYVFhaOTFJNTZRUlJn?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiW0FVX3lxTE1RdV9pa3ZIMmpRWnFlcXRaeTRnSy1zZUp0enVScm1nc0hMX3UwTEdEOG9oQy00UUJiSUR4WENleElGQVVmLXh3ZE10b09nQWphT0IzNHNJb0h3Q0E?oc=5</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr"/>
@@ -961,12 +961,12 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -981,12 +981,12 @@
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>UAE extends small business tax relief until 2029 - theaccountant-online.com</t>
+          <t>FTA Directive No. 5 of 2026 - Crowe</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>News — UAE E-Invoicing</t>
+          <t>News — UAE VAT</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -996,7 +996,7 @@
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxOMTA1XzlxbnpmYjNMcU01VXV1RjdMOHFuMi1CSVNMYXlaNW9kb2ZMSXZXOEZ1dDlqbmRLR2hXQjNrMDdlaU4teDVRTG1CMmJsY0lDU3V0SWxRZE4tWXZXbV9pR2o5THFMREVyZ3VpY1pTYVhFeUJza1MwOWtVYXB1ckwxQlBRdVF6eURUUHlkblhUNnNoQ3c?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiVkFVX3lxTE40S0RnRzF2d1dBSmNHdkNNQXZQQmlOYWNOSk5OWnlVNUN3ZDB5UHBUV29RXzNvaF9pVFNQZ2FwTUdocGhxMXp1T3gxMUFycGNESFA1bXNR?oc=5</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr"/>
@@ -1006,12 +1006,12 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -1026,12 +1026,12 @@
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>Sovos Announces 2026 Partner of the Year Award Winners, Recognizing Excellence in Strategic Collaboration and Innovation - Business Wire</t>
+          <t>Digital currency and VAT: New UAE rules for businesses to consider - thenationalnews.com</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>News — UAE E-Invoicing</t>
+          <t>News — UAE VAT</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -1041,7 +1041,7 @@
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMihwJBVV95cUxQRzJIdmQ3VjZqenlUTldPal9HNXdxdTJibTJHWFBhMVBMTWcxbm0yeUhJYzVLd0Z3Yl9pdE1LQzREWm13dXE4ZG1abDFuRkZIdHhIcm4zYXVoOXZIS01KNW5xRU04SUVwMlRnZlBxb3BYQkJMQ01CeXhabEI5U1VfSlpad0ROaVNnTUVnUll2WFhwMkxUa2tidGRxTDlMRm93SlAxVkNoWW84Zk1oeFFoNVdnOWRBZERIZzNSdnVDMGpHZ0MzSXlxZ1JXc2hodEY0aXNoRkNBRldSOGdxSkowdmFoTEplTjBtOUVfeWFtNmpzeDZtR3J2bVk4UWthWFR5VjJRbEM2NA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiugFBVV95cUxQamI1MElzOEtNS1ZjVWR3VGpjZjNUZjBXbjQwZkJIZ3AwOFVqckl0WWFQN2JpaEg5XzRTUTBVMDFOeVhMaUZxYW9GUnBFNW55WnhKd2ZKOVZoekRBWUNqQkp3dGFPZ2JQcWY5SjVlRUJuTURfcVN5aUNXVmthdUh4cHlJbFNHN3lyT1VTU2l2Nk92U09JZFh3eXp0c29jTlJNZW1VLTZBR2h5WmdBTjFuNGczZkZwdDY1QWc?oc=5</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr"/>
@@ -1051,12 +1051,12 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -1071,12 +1071,12 @@
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>UAE E Invoicing Guidelines Updated to Version 1.1 - Crowe</t>
+          <t>Air India turbulence injures passengers on Phuket-Delhi flight - Gulf Business</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>News — UAE E-Invoicing</t>
+          <t>News — UAE Corporate Tax</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -1086,7 +1086,7 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMigAFBVV95cUxQOGUxa2xtLVY1ejE0azVCMEZSa3lxNHZmajhUdzh5LTQ5NGRqVk5oenBzNmJUSk44X1B0elZ5aDI5YVl4VHpLb2RzdEFRYW9IVmR5dHpOaE1JbWVoNzdvQVpsR0xIalA1MHBaR1NNOVpVSHUyX2t4R0dIVmZiWHlXWg?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxOUk92b3hCQVZybGNndXNJOF9ZX0Z3TGl5NnRuXzE5NlBRb3czZXM2SkxXb3ZQSGNOdGo2a2U2b040ZVFDcFBqbzdvaFFZaVdBbFgwQkJOOEhDNzF6VXY1OU9Ca2t2Z1ZnQlhscXNXTVhDaWY3b2lvMUlEWFhkXzVxaDR3b191OUx2aTVKcEttYkFGTjRzRVpnbFJvLUZhYmNLTFJJNg?oc=5</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr"/>
@@ -1096,17 +1096,17 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>VAT, E-Invoicing</t>
+          <t>Corporate Tax</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
@@ -1116,12 +1116,12 @@
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>Congo Republic e-invoicing launched - vatcalc.com</t>
+          <t>UAE Business: UAE extends small business relief for corporate tax until December 2029 - Gulf Daily News</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>News — UAE E-Invoicing</t>
+          <t>News — UAE Corporate Tax</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -1131,7 +1131,7 @@
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMijgFBVV95cUxOLTlBQUhqTDJya1ZpUmx5Y0lPRlRHb0VpWW5GYWVBc1JkTGRFbFl0b3N5UGJSdEdXRmwxdld1RlhqSWVremtIU1pWSHNXb2ROejA2TzJYcF9RX29TQVN1akJ5d0cxWFplcmJPYUJTRDgzU2FzenRzMzJldUsyaE9rbzlVUmJMSEc5M1pzSGtR?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxNVm43RXV5MWlfOTE5TjdqQjhtd3pzUnRIdmJycExNbXV6REpoRjQ5MlNiRENNemM5SG5VbUhJbnVXenhQXzFhRGgtNXE3QjRWWHhCcTJsZ0lfUW5ZTWNWcjdZQnZSSDM0VVdvVDY0ejBPMklPTUkzdTdXX090b1RQY21nbmdUQUtuZG42RHBxRWdCb05xNkdBT2xUVk1SNWN0cG1NbnhKNlBxSl96T3BzOU91cw?oc=5</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr"/>
@@ -1141,17 +1141,17 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Corporate Tax</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
@@ -1161,12 +1161,12 @@
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>Corporate Governance in the UAE - Crowe</t>
+          <t>UAE extends corporate tax relief for small businesses until 2029 - Khaleej Times</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>News — UAE Transfer Pricing</t>
+          <t>News — UAE Corporate Tax</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -1176,7 +1176,7 @@
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMibkFVX3lxTE4weWRYb0VETFpvMjdhUG9BbU5Wb2JXbzNkLVpxSC1VZHhwYjMwT0F2OFNvQkJNQTFkOG1OamVFZWU0NWpVN3hHb0lldkJWLV9GeThwSjdzNlpnQXp0VDdQbkpnSWFFU3lacVJOeXl3?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxNMDNwUlhpclFxaFJkdkkzR0s5MVh4WHZOUDdfZzZtNTBFb2RIcklxMF91Tkp2NGRxRlZMM3BubEZGc0g5LXpsQUhHQy01eGcxTllzc1k1S1NqeFMtYXM4YlBmREttNlhsS0hmd2JXN0l2UjFEQ3B5M1pfRTVpOGw0Z1pPMTNHd0tHQ25ZNjNGZmVaZnhzZUJueE9sQ2dNNGVaUDVjTdIBrAFBVV95cUxNbWJjeHFtRU9DbExyNHRRY1NEUXB2WnZRZ1V2TlFhQ010T3RhSmptR2ItaDhxVnEta0NITUJyS3ppaGgyQ2FkclQwRFhCaWNnLUhNb21YaDVGLWZZNThic2hpN0MzNTI4cXI3RjYtLVUzN3VHanJUUHdYaEFRWUlvS2w5UVdja3pwd1Q4c2pXWHVPZ0xZVmFCcE43eWl1bG10N0s4UXdpVUhpU0tH?oc=5</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr"/>
@@ -1186,17 +1186,17 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Corporate Tax</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
@@ -1206,12 +1206,12 @@
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>Shopping online in the UAE? Tourists can now claim tax refunds on Noon orders - The Global Filipino Magazine</t>
+          <t>UAE extends corporate tax relief for small businesses until 2029 - thenationalnews.com</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>News — UAE VAT</t>
+          <t>News — UAE Corporate Tax</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
@@ -1221,7 +1221,7 @@
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxNa1BKRVpJRVZCZm5VNVp2d3h4Rl92ejg0aml0Qy1pTUotYTZ4ZHlaeURMcnRacE9Zc0J2TWt4VktTQWdFV3BlNXBzWmlfMXFEZFRiYWRIMmV3X3ItaWc0T3pzOG52THI4c1RQaDY1RWdNbXItTTUtdlFTS1d6SUpZTVlXM2lOTWtLWXF6TGNSRE9OWkJQSUs3UXFoSEtOa2NpNEJLeTFOektldFVUVHk4cFJCSE5Qdw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiwwFBVV95cUxQOFMwcEtFYkFkbWxMRnBqX3Y1M2ZOcnJ4Q1FzTHg2b1NDYnU3dzVWMmMycVdhNzJSbTZhaTZ1bjRpN3RYcm9Gb3VIOUxydjN6anFTMU12SHNNcmt1YkhwSk1RVTV6Yk1yS0wtNm9PbVZLNkxmTVRNd3hEOW1xbXdnTlBiX0VJWWhINEw5MHc1eEk4UHhFZHFOZ04zcnZERDZhLXZJQ0VGWS15N080ZXBQYVhDMFU2al9wN1NlNXN2RnFaZEU?oc=5</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr"/>
@@ -1236,7 +1236,7 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -1251,12 +1251,12 @@
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>Number of retail outlets connected to Digital Tourist VAT Refund System reaches more than 19,300 - Big News Network.com</t>
+          <t>September 1 change: UAE announces new excise price rule for electronic smoking products - Gulf Business</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>News — UAE VAT</t>
+          <t>News — FTA Announcements</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -1266,7 +1266,7 @@
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi2AFBVV95cUxNUjRVVzdLOXJQTXpUZDhqeWlQNDAwVDV2ZmJqd3h4cW5ZbXc0cHEzZGJBSWlLOTk0ZlFFbXlVSThCUEtxcGFqUHYzSlRmeXF0bC1XQ1J3VVhKUUkzeVBfNTc4cmQwNmlRYldwUU01YXpmc0pxT0daNWRpRUwtM0N3MlBBR09rRldZZlA5bXVJOXVTcVZSeE5ldWRHSWhna0ZfTTNwZWEwODlFTXRRYnRhOVJVcHJ3dDRuSnZtQlBhc0NMa2dhSzk4b1lBWEx5Uk5Ld2RMaFdmNUY?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiwAFBVV95cUxNMXNESjR5VDVIQ0Qwb0xKUk1xRlhaTmV2RjNfdVpGaDZZYk0wcjdSbC1RRHBUNkRRaGpNOS1mSjR1blVVRHJ6MzdLeUZXM1lMWURyX21CS25DZFN3engwRWZCOFFLUDJydEEwX0pSa1lLSlNqbVlhdk9pNmtvLUh1QzFubU9RVENUNEl3QVdLc2FkRUV6TGFjZmJwLUtiUVd5dlhjVW1SLU43WFI4eGNfZkJCTXBNaEQySVR3QjZuazA?oc=5</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr"/>
@@ -1281,12 +1281,12 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>VAT</t>
+          <t>Corporate Tax</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
@@ -1296,12 +1296,12 @@
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>UAE tourists can claim VAT refunds at 19,340 stores and on Noon purchases - Gulf News</t>
+          <t>UAE small businesses claiming tax relief must still file corporate tax returns - Emirates 24|7</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>News — UAE VAT</t>
+          <t>News — FTA Announcements</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
@@ -1311,7 +1311,7 @@
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxQeDRPcDE4QjJaSFU3Qm1wRGVaWXl6cjY2c3YyVDF3TmtqN1RYMkh0WDdoSm56QmlXU21xSllRQWt4WHNFU09vUWZpTEd3dVVMb0UxNy0yZG1ucUF6aXhIZ2dWVXpkVjVqa2hHUGN3VHNZWEticFZMXzNfb2NzaVpwOFFkOVAtNDhBY0xjSUo3bkh0WUg2ZEJ4Q0JDU05Td0FTLWlUWXNfN2JKeGJsTEg3NGFDMzNwT21JZTFGT0V30gHQAUFVX3lxTE9wdElvSG52YzNWWUt6WGJaRkp0LXpmVHpQTFV4WHczVkQtOUhOMWpqRzd2UjgyQjNOSWdMT3QwM1luZzdtNWhXdU91R2lqS0FKcG1hUGExZ1QxWG1SSUo2cWZSWll0bjdpQ2pBOXFjTUMxcjJma0RraGlVbjNjajZRM0h4OVZfM0FUQXNERTQzQm1TS29QVjdiQzM2T19naktoTXhfQ1pvNmx4U2IxVkkxUWF5QmZ4QUxmMXB2bFVvR2RVWm10bjE2SlNaRzJ2VEU?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxOLXJ6YVV3T2dXazExeU04V09UYlk3NmtYT2d3Z2t1X2RPckN0RjVQZE9oNTljdi1rUUlzTDlMalotZ1JWRS03TWVFWlVVS1hyMVlDUEsxYWQ3RWgtdTdUNzVaZjE5WlhVVUhJcjkyaDFVa28yeEN2ejAtVG43dnduV2NDa0k4czRLby1sU2w2ZHZTcGtPZmpiTjRYWXB2VUExMnhreUktUDBZSkZ4LUxZYW9TYXRJc2s0U1QyMtIB1wFBVV95cUxPNWVmQzRQOEJkZnBCZVFDblE2dkFlX1hGNWlnalJBVk5QREJoU0ZvMXZIM1JJYXdLb2lQZFNnejliekY3Y29nN0tLdTUxQ0h0SUFaSVlpOWhuX3dVaHdjX3NPM1pkd2xlVDRMT1VmTHJ4QV9PbmpWRmVHRFpHZ1lyUF9ZWEJTcFJ2LS1QX0hEa0Y3dnJ4S054S211cWRMWWlHVVd2V19wQnhGa2JVR1ZxSFVNVWJMejdESlFZSkxUMGYwQUlyQkpueDlwb2dJYnlqQnZGNklscw?oc=5</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr"/>
@@ -1326,12 +1326,12 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>VAT</t>
+          <t>Corporate Tax</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
@@ -1341,12 +1341,12 @@
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>Retail outlets linked to UAE's Digital Tourist VAT Refund System exceed 19,300 - Emirates 24|7</t>
+          <t>UAE releases registration requirements for domestic minimum top-up tax - kpmg.com</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>News — UAE VAT</t>
+          <t>News — FTA Announcements</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -1356,7 +1356,7 @@
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiugFBVV95cUxOcXRBMGsxX1Q5SkJXcEFwWnV3c0VVc19jUnRkWU5yMVlPelltaEhvOWNLcEJxYi1KUExWMVlmZE1FOExZYklsRHU4N3lQZGppMDRnYUFaRU1OWHdwaVpiWWowOENidVJjbDFPeTQyQklzOGM5bXhQbDJrRFg2TkR6bUplTzJNZzl2M3dJT2FEeHVTTVNtTml6UEdoZUFDcVRCZWFHMGg1ejZoSWI1UWFCLV9zREotcmF3V0HSAdQBQVVfeXFMT3Q0RFN0V3FRSlNWV20tMm5hY1N5VHBVWmxzdnZGVXIwZU92VTZVRDVUVkRZM0Q1U1ZNZzFRcFlEWTc2ckk0UjZhcEN4YmZIZndTd284ZDQ3Z2Z4OS1mVGFUX2RwRzgyMWViTjEyQ19wdUxucXEtZWtFRm5tOWpId1VYYlRmd1Rkc2tlb3Q3THR0THZxZWt3Q1ZyTGVvZ2hUUzZPeTBPSzlER3FXR0ZvUnJiWk5vdlpwYlYxdmZjZnNTVEQxM3hSY1pyTGV5Qkk2d2lrejQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxPaGJWUy1MU0VZdmd3LTVPTmw0bDYtWlF5a3JCVkFwVnhJRUkxVkdEWUE4X1VZLXg0Tkg4YTlLWHhoOUJYVzJqR3lzUE5Pa1RpSWtjdkRDQ09UeDBoQ3Y2bGlLbkhzTXZ2WlNJeGFSLXNqRUZyRnBfNV9Mbk5UY25hdVZ6VWM2cWRYOEt4bUlnWV9QYkQtOWZudGJaV0ZJZDRVY2JGbTY1T1JTYVhyTGhEdlVuQzlzZkN6ZC1VRQ?oc=5</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr"/>
@@ -1371,12 +1371,12 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>VAT</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
@@ -1386,12 +1386,12 @@
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>Indians, Russians, Turks top list of tourists claiming the most VAT refunds in UAE - khaleejtimes.com</t>
+          <t>UAE Digital Economy: Why Trust, Not Speed, Now Wins The Race - Menafn</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>News — UAE VAT</t>
+          <t>News — UAE E-Invoicing</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -1401,7 +1401,7 @@
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiugFBVV95cUxPek9sY1dJUkpRblhiYnJDdDExOW1yREdXd1oyZ1Yxb0FnZlBYNTd3SUxGWnVMenlZVGlqRlIxLUszNk1Jd3BpcF9rVE9XLVF1OWdhY01fd0gteTJFRkVJLVREMjl4ZVRGZHJacUxJREpRN3UxdHFncGhITEQ0MnUzTkhKY2FSZnBnaFUzZDEyRnZOdG1hOWVFX2FLNG9Ca1lGekQzcllxd0FqTUhvTTRZM3MxcElQV0JaMWfSAcIBQVVfeXFMT2FPTEx4WGUzNUNhZWdBa1MzVU5GN1p3SkRwM0o5TWlqenhqVTNhR1Z0bThyN0laMS1tOUhfaG1qMmZpQi1pT3lTNEhKT2l3SklKZ1E3MXkyYVBrMnUwOTh1Y2RxSkFISUdlT1B6Qm1tTV9CUV9YM0xwcTJ2NzVmWUcxaFJ2YzhYeVBjZG1WSG9vcVc2N2tqRzNreHFwWVpaaUdncndzVEVLaE8zeHczU0Jvdl9FazU2NE1CNWZqQmZmekE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMikAFBVV95cUxNbi1OcWZwSTNNYjBRZkJWS1FodlVGTG5oZHB1T3Q2cGRqazRiZGQzeUtlOVB3VXlhNUM1TnhSdW1MVS1uSng1dGFmTlAzb3ZMNXlod0c5bWo2RkdOTW1idm9JQ3dQNTM5Z3FvZl96WlNuVVh4Mmx5NGFNWXBHVFZoWnUyQU9WT01idllWclJqTXE?oc=5</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr"/>
@@ -1416,7 +1416,7 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -1431,12 +1431,12 @@
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>Tourists can now claim VAT refunds at 19,300 retail outlets across the UAE - Gulf Business</t>
+          <t>Ministry of Finance sets e-cigarette liquid excise price - Sharjah24</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>News — UAE VAT</t>
+          <t>News — UAE E-Invoicing</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -1446,7 +1446,7 @@
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxQV2tyUkVhVzNVUlZ0QW9LdW5PWV9OTEVSN1FHU2c0Um9qbTRDNXFIdmZUaERGcDFPUkkyTVpzWXBQblJHb1VzVERybTh5WkIzcnRoRFo1ZVBicVRMQXpFZXB3VVJRQVZ6UDNNZDItT1RuTXcxYWxtSU1PaGlPNTFNUnpzLXBGX2QxSy1WVjU4alg4Q0dEWmY4WFZ6cEt1a1FZQXpRODFFN0xRT3VwSWFfNw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiWkFVX3lxTFBGY1BCNkVheXBxM3RBdWlPNXVULWVaaWdWM3RWWU9JSWI2T3JVMGlMdl94Ync5ekFqdGU1SzAxeEMwaUhJR1hTejhVTFo4blI2Y1d5QzZUaVgwUQ?oc=5</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr"/>
@@ -1461,12 +1461,12 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>VAT</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
@@ -1476,12 +1476,12 @@
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>UAE tourists can now claim VAT refunds on eligible Noon online shopping purchases - Arabian Business</t>
+          <t>CBUAE injects more liquidity into the banking system - EnterpriseAM</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>News — UAE VAT</t>
+          <t>News — UAE E-Invoicing</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
@@ -1491,7 +1491,7 @@
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxNSk0xOTlEQk5DQm4tczlCUE1jZ1dmamdsaUQ2TUYwWnlNd2JHMjhhVXZVUF8wNGpSVUFRNXhvU01pY01FMlUwWEt0anFyS3Q3QS0wa3BjZE1YLWtkWkpYeUJxVmlaSUhQM0Z3Mk9odUFYenhNRnBZeUkyQ0doNWJ2VGUySGY2dG9kMnlJaWhuWEMzb25aWjA1VXZkLWRwelk1MXJjbjBrV2F1Z29KZTJ3?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxPRVF2amFoSUlsRENGenUxcUlxRU9NeU9QWlJhUkExb1k0cExublF1YUdrM2dJc0FySm9zQmgyQUtKU092bkpYT1I1bUhaMkxGR2o2SFVnckhIR2d4RGQzOUJnb19tZERINThyZ0NrQ1A0WUttandLcmN0QUlUaTFVZ1djMnUxdEp4SmNGMjM1Zl9HX1k?oc=5</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr"/>
@@ -1506,12 +1506,12 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>VAT</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -1521,12 +1521,12 @@
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>FTA issues five binding VAT directives on tax transactions - kpmg.com</t>
+          <t>The Taxation Society partners with Tally Solutions to strengthen UAE's finance and tax professional community - khaleejtimes.com</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>News — UAE VAT</t>
+          <t>News — UAE E-Invoicing</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -1536,7 +1536,7 @@
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxQQXptRUZOQlpWYUZiNzd1QThPVDhlUGM3TF9PU3NKZjUyS2lucEZLUUFKZFpfZVhXLWxteTBKbU1OVEU1WXdPVlViT2ZBb2h5dmlHa0Z2bjd0SzMxa1p6TzF0ajhuVFVSaUpkczUxd1lzeGVCeDNwRnpPbXJVNVNGWHB4UTcwR2dCYTJoWTVSYkJGQmxRZE42cXNmOExtclgxR28tUUdYVFRzaE92?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi4gFBVV95cUxNMXRpRGhpQXJvUkZhQU1IcTF6Z0JtLW16cTQ1d24zZWlwQTlPMHNCeG8tY0NLc1JGcXdjT2g5V01YM3hOVmtZYzBJeThiR3hhSDRpdGdwaDhsVC1WMDFTSWN0SWdhc3hiWTRSQmV0blZEZkowYWdoSU1BaUJ6Y01ZZ2ZrWlNRc2JtUllnc0huTF92aWdmbEp4bTRvRV9fN2xTU2dmMjdLSk43ZlFlcEtuWTBKQXdFTU5pMlRnWE55VFBwcTc0STRtcFluS3Ffek1oM2NRQ1dYemVkTktESkJRSVJ30gHqAUFVX3lxTE85ZnVhMjFKMWdhenV1YlFiRGtpVTBIdjRvLVNLRFBjTHBPUnVfeG5sUGxIcWVlSlhUTEVibFV2UXdWbEg5TGNmS3hBYnczSEctV3BBT2pZT3dpcDJUeGczWE9xQ1dweV9hc1hwQnhHQkFWUDRrb0FzV0tVdmZhZ0pLZC14YlVJZjBYQmcwbUZWeG55dnhpOFliT0wxYkQ0bzl1VEhiVUpQNjQ4TVN0bFhPRERROXB5NUZZQ0VRS08tY0VmSDdLRFQzMHZ0dEZtamJ5dmp1OGZ6SmNxQjZrck8wRWs2U1A0TFJZdw?oc=5</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr"/>
@@ -1566,12 +1566,12 @@
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>UAE extends Corporate Tax Small Business Relief until end of 2029 - travelsdubai.com</t>
+          <t>MoF extends Small Business Relief for corporate tax until end-2029 - Sharjah24</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>News — UAE Corporate Tax</t>
+          <t>News — UAE E-Invoicing</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
@@ -1581,7 +1581,7 @@
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMingFBVV95cUxOYzFrN28yN3RDREhxYV9CVHl3UGU1NlpvSFJqaHJGWVpraVhEOEtqTnZVQk1OTjVjX1djWENocHdtYy1WY1dBSHZncjg3aGxWOXlwcFktaVVxYzBmZllLbzBaLUUxSEpyNW1HX3V5MG9YMWhTcjNfcnZxQ1JKRHZkMjlYSjlmUHk1SGFEYy0tYmlqWE96ajBqUnNSS19TUQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiW0FVX3lxTFA4N01YTUZ2UGRGVWdDQ3JDM3JLYWJDanVuckdCLVhuQUdqUFo3clA1cGRoTUtubWNpQ0dTOUFSQk5jYzdGcVFYNkNpQjF4ckFVZ2pBc0FXM1Ffa0k?oc=5</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr"/>
@@ -1596,12 +1596,12 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>VAT</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -1611,12 +1611,12 @@
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>UAE seizes 3.58 million non-compliant excise goods - Gulf News</t>
+          <t>Northern Emirates’ property markets cool off + Sidara locks in USD 1.35 bn in firepower - EnterpriseAM</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>News — UAE Corporate Tax</t>
+          <t>News — UAE E-Invoicing</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
@@ -1626,7 +1626,7 @@
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMipwFBVV95cUxOOF9vUDk3UXlsY19FUWtOOEJ2V3Awam9fY09zeS1seXpTUUt2Y05TQlVUVjlwYlVuX2hRN3JBM095eTlqZ3pxWWx5ZWJzUzV1bGdCQ21JMzd1bjRIMGRMdHpiZWVOM1lmOVdtSXlicW4wYUNoYjMySjFTNl9OTnRvYWZycGdhODlTcU9sQUpwUEdJcnltNF9nSXpBWkpJbjF0VG1qeVJqTdIBugFBVV95cUxPMDVISGFVMTVqWFFiS0VMTmlzZzlyWXRVUl9BTjBGaWgtS21lN05BdlppYlVNQkNtYmZWaHRIczNlSWRmbXBBdG9zamlobjFhTFh6R2lYZFJ1RUtKWGZqOWpNd21LTmNxaUF1SjVIUm9UNjF6cmwxUGY2ZHFIVHBFdVJNMXcyeFp3dUZ2V1hpVmtnRmZOY29nLWNWQmxsQ0tHUzd0RjRyRUlZeW1adThtZEpPVl9KT1pFRUE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxOMDUxZXd1MElSNXdaNDByLW9jbHFIenJCY21PRnhPMUx4YkdyZ1FMREVxenNWZWZUY2p3MHQ5V2xUQmswZ1RuV1g3Q3RHUzdvOFhvOGpST2diQWIwOXFBeXdzc1lYRl9FRDIxdjBjUVR3Y2VEcUdIWXB0amg4YW5qbklORzFMS3J4VUZGelkybDVZcXc0VHlNck4zTXdjR1N1UzZmSk9vSFFoMDJMVENKMFVlWEdvUTEwZFhiZmdn?oc=5</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr"/>
@@ -1641,12 +1641,12 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Corporate Tax</t>
+          <t>E-Invoicing</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
@@ -1656,12 +1656,12 @@
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>UAE Extends Small Business Relief for Corporate Tax to 2029 - tbreak.com</t>
+          <t>ClearTax urges UAE businesses to prioritise execution assurance as e-invoicing decisions gather pace - Gulf News</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>News — UAE Corporate Tax</t>
+          <t>News — UAE E-Invoicing</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
@@ -1671,7 +1671,7 @@
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMifEFVX3lxTE9icS1QSXhYc09ROHVJdzRtdXJTMEdLa0o5Mm5TZ3VxR002a3lTeFR5anZqRmNtcVEyQWxfQ050UFVOZnFBcFdwT1VoNGlVZU9xYkY2WkM5SlpSSnp6QkpHck5rTUxqOXNjNjM0UmFTQkFfOXZySFFON1pCSXc?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi6wFBVV95cUxPTG13TFpCRmpaaWU3ZGxsVEtqakxUUXhSc0ltWUZfOEUyWTcxWGhOZ2doazNZY1V2LWFnSlp0NHpHTXN4emN6TzFWbGlXT09xU0Q3X25BTmpBVVl0Nl9XMFdRUE9HMy1BU3BMRDFIZ1RITkw4d3BSanluZGFHal9CM3h5dDNtTlBtUG9LYXZZWkhILVZhdUpKTHhUd2lMWmVOdVJrREx4UUF4WjNvTW5hSmtBVjVyQVBpblVKa1hKbjhxRTNUVmpUMVpXOFFJSWx1NUZWUWFMYlY2ZjA2Nml6OGV6X2ZGcVhkQkQ00gH-AUFVX3lxTE12b1Q4Qjd0Rks3U1hqOC1GVTZ5RXRUOXB6eVdVd3RMTEV5Q1pRYVRrc19GaG1qY3FXRGhqMkN3N3c2emJyeTFWbEU2QkRSMHR5aWFzNlctUi1mdi1vamRHMHZoWFZlQlRCbEhrT3BLSXlsTXRfYjY4QjVHblFRU0JnZVhlam4xNEF6d0hQVUtmTHFoYnktSW5LS3dqU2VleEh4azlObnoyUTNPd2E0RWc4U0ZhMkRoc1J1c2R6VGJhc1lSYTF0cjhzdnY0Q0tvYk81YnY5UE5CdnBXZTVNQXE4UlZwMkFjbUREaEtRNlF2MWJYVFhaOTFJNTZRUlJn?oc=5</t>
         </is>
       </c>
       <c r="I27" s="2" t="inlineStr"/>
@@ -1691,7 +1691,7 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Corporate Tax</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
@@ -1701,12 +1701,12 @@
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>UAE extends corporate tax relief for small businesses until end of 2029 - Gulf News</t>
+          <t>UAE extends small business tax relief until 2029 - theaccountant-online.com</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>News — UAE Corporate Tax</t>
+          <t>News — UAE E-Invoicing</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
@@ -1716,7 +1716,7 @@
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMixgFBVV95cUxNNEo4Tm9qN1dERmwzZ0tMR0ZOSUVQTkpOTTNiTDc1U2VaSTkyRkExekRzRjUzb2xrelYzV0oydU1qS2JCbHJXd1hxeWhPdmtUN1UtcXRCOHZpSXBxMlBMdFRKbDNxYlNFaVdwRXROTUVxWC1tZUpObDVIZzNVUDEzSUZpNkIxN3ctTDRNWU9xOUx6QXZieFdVV1hkNHhlcldHUzY5b21BZ1J2VTVhMlN2a1V5V1dJRkw1OTItdWo5Qzk5N2lPX1HSAdgBQVVfeXFMTmRQM08wYWhkelVySDhudHZWLWQyZ2lyUG9TNEJhWVV6ejAybDV6QXdvUFR5ZndxZldxWHVDMjRKVm1Ndm0yeE1HZHo1LXoyVFBzMkhuUDZESEw5RUFIaWlfNEdObjNxRlc4VFpOZVQ3RDhhellsdEpYN3pLVzl1d1Fva3R0RWpDb0d5cVN0Z3I3emowS2tNbkplWTh1Z2NvVkRMd0R3STNWV3hrUVFtd3hxdjQxWjI2ZU4wVE9JTzlsWVUwYXlPTmU4YWJmazMxQk93MHVHbGZE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxOMTA1XzlxbnpmYjNMcU01VXV1RjdMOHFuMi1CSVNMYXlaNW9kb2ZMSXZXOEZ1dDlqbmRLR2hXQjNrMDdlaU4teDVRTG1CMmJsY0lDU3V0SWxRZE4tWXZXbV9pR2o5THFMREVyZ3VpY1pTYVhFeUJza1MwOWtVYXB1ckwxQlBRdVF6eURUUHlkblhUNnNoQ3c?oc=5</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr"/>
@@ -1731,12 +1731,12 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Corporate Tax</t>
+          <t>VAT</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
@@ -1746,12 +1746,12 @@
       </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
-          <t>Small businesses in UAE urged to file corporate tax returns before deadline, says FTA - khaleejtimes.com</t>
+          <t>Sovos Announces 2026 Partner of the Year Award Winners, Recognizing Excellence in Strategic Collaboration and Innovation - Business Wire</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>News — UAE Corporate Tax</t>
+          <t>News — UAE E-Invoicing</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
@@ -1761,7 +1761,7 @@
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxOWnJlYmRmRm4xdy0xZ0toMUNUbnhTd3A5UW1pVzhFeXhIM2txamo4NU5qYVYwZGlQcEYwLTJhelBkOEdHajRYSE5PRnZtdmxGWmc0R2JlUVk0eVc0aW53NzdlM08zeWFzTUNocU9UcnY3UTNhTHVzZHhjRXFPZ0ZMMHMyRExEcjFiVVhKVzMxYk9FSHUxdERQRnUyZlJLWXA0ZVHSAaoBQVVfeXFMT3BwVV9lZzBQRTFjWUNVNEFzaUlhOUJuTHByVVRhdjRTbjdpajdOTjRtc2hfOEotMWlSb0FvX1F3azI2czNjMHREWnRJbFptM0F5ZHJkWUFsMW5fMDBsNU1YODgzT2VkMWZacU51MzkxaHJ0S216TF9UR241SnM0OVo2eHlDM0F6V2VfbUt4elZfZVBub2pLNW5fazhqV1hNUnBzRmkxS0NUQVE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMihwJBVV95cUxQRzJIdmQ3VjZqenlUTldPal9HNXdxdTJibTJHWFBhMVBMTWcxbm0yeUhJYzVLd0Z3Yl9pdE1LQzREWm13dXE4ZG1abDFuRkZIdHhIcm4zYXVoOXZIS01KNW5xRU04SUVwMlRnZlBxb3BYQkJMQ01CeXhabEI5U1VfSlpad0ROaVNnTUVnUll2WFhwMkxUa2tidGRxTDlMRm93SlAxVkNoWW84Zk1oeFFoNVdnOWRBZERIZzNSdnVDMGpHZ0MzSXlxZ1JXc2hodEY0aXNoRkNBRldSOGdxSkowdmFoTEplTjBtOUVfeWFtNmpzeDZtR3J2bVk4UWthWFR5VjJRbEM2NA?oc=5</t>
         </is>
       </c>
       <c r="I29" s="2" t="inlineStr"/>
@@ -1781,7 +1781,7 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Corporate Tax</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
@@ -1791,12 +1791,12 @@
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>UAE extends Corporate Tax relief until 2029 for businesses earning up to $817,000 - Arabian Business</t>
+          <t>UAE E Invoicing Guidelines Updated to Version 1.1 - Crowe</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>News — UAE Corporate Tax</t>
+          <t>News — UAE E-Invoicing</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -1806,7 +1806,7 @@
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMieEFVX3lxTE5SM3FoRTVUSmJwTlpLbi1vOGFPM3RPcXpraXlCUG9iQlhuUUJ2MGRCczd6aDM0MFFNWS0yS2tNNVIxYjd2Y3AxWExhUnJNcHNXT3dLdGhyV2FBQUQwbmZ3YjRZc3NXTkNoLU5HTFRkTWRkSlZ6TEtHbg?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMigAFBVV95cUxQOGUxa2xtLVY1ejE0azVCMEZSa3lxNHZmajhUdzh5LTQ5NGRqVk5oenBzNmJUSk44X1B0elZ5aDI5YVl4VHpLb2RzdEFRYW9IVmR5dHpOaE1JbWVoNzdvQVpsR0xIalA1MHBaR1NNOVpVSHUyX2t4R0dIVmZiWHlXWg?oc=5</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr"/>
@@ -1821,12 +1821,12 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Corporate Tax</t>
+          <t>VAT, E-Invoicing</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
@@ -1836,12 +1836,12 @@
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>Ministry of Finance announces extension of small business relief for corporate tax purposes until 31 December 2029 - Zawya</t>
+          <t>Congo Republic e-invoicing launched - vatcalc.com</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>News — UAE Corporate Tax</t>
+          <t>News — UAE E-Invoicing</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
@@ -1851,7 +1851,7 @@
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMihwJBVV95cUxOWVAwdTI2R09XSWRHaFNWYkNGdUJsSTNnaGpRandNeklubW8zM2h3VkNIcmRiQTVrZUxlSnhydWtqUGVTRS1vYVVQWWJfY2swUzhYOFJrdHVCQTlvTk1LNVBfWjBPbHZxWVU5Q0xQVWFHbTlLYlE0ek1aWFhqaUF3dDlTY2p2T0dtV3gzSXhaWkdFdWFBejA5ZkhDSkVPanZUWDk0d1oxNlJOUkNxMER2M1oyc3Nla2NnUW9WYmFRS04zeGlCcjQ1YVNZT2ZraU5EN0h2ZWRDaklZTjFQUklLWmRGRVFkUjhKUjBybHA5UktLZHFiVnUtOFpuNmhSZ0o3YVV3eld3WQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMijgFBVV95cUxOLTlBQUhqTDJya1ZpUmx5Y0lPRlRHb0VpWW5GYWVBc1JkTGRFbFl0b3N5UGJSdEdXRmwxdld1RlhqSWVremtIU1pWSHNXb2ROejA2TzJYcF9RX29TQVN1akJ5d0cxWFplcmJPYUJTRDgzU2FzenRzMzJldUsyaE9rbzlVUmJMSEc5M1pzSGtR?oc=5</t>
         </is>
       </c>
       <c r="I31" s="2" t="inlineStr"/>
@@ -1866,12 +1866,12 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Corporate Tax</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
@@ -1881,12 +1881,12 @@
       </c>
       <c r="E32" s="3" t="inlineStr">
         <is>
-          <t>FTA reminds small businesses to file corporate tax returns - Sharjah24</t>
+          <t>Corporate Governance in the UAE - Crowe</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>News — UAE Corporate Tax</t>
+          <t>News — UAE Transfer Pricing</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
@@ -1896,7 +1896,7 @@
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiW0FVX3lxTE5NZ1VTdFlkVERkd0pETmFiVUQzZzEySVNaeWFyV2N3MHdhSWZreEZnUDFCYXhiWGtCOVVxMFdWUzhDa3JCU1czenE3QzJzaG0tNU5iMkFmRFRsTUU?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMibkFVX3lxTE4weWRYb0VETFpvMjdhUG9BbU5Wb2JXbzNkLVpxSC1VZHhwYjMwT0F2OFNvQkJNQTFkOG1OamVFZWU0NWpVN3hHb0lldkJWLV9GeThwSjdzNlpnQXp0VDdQbkpnSWFFU3lacVJOeXl3?oc=5</t>
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr"/>
@@ -1911,12 +1911,12 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Corporate Tax</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
@@ -1926,12 +1926,12 @@
       </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
-          <t>UAE extends small business relief for corporate tax until December 2029 - TradeArabia</t>
+          <t>Shopping online in the UAE? Tourists can now claim tax refunds on Noon orders - The Global Filipino Magazine</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>News — UAE Corporate Tax</t>
+          <t>News — UAE VAT</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
@@ -1941,7 +1941,7 @@
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxOc3RJWW11LUNyUERIeHh0dTVRVFJySzBoWVB0N1RCdVNpTVpORW03RkVXaG1pdk5HbWJfTDUzYXRIellIdlo4dVBXcXpuZHNrQXZRMk5MMGF1UkpqbGRTbXZRekZTYkU3cHpsdmJHdTVRdFFxSE1aSzZxWW1rb0RuT1RNZzVOWG91OGVTcFZVUGFVLWRUY3JsRnEtYkR4WUJjWnp6NkljSUd2NExsdUYtVA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxNa1BKRVpJRVZCZm5VNVp2d3h4Rl92ejg0aml0Qy1pTUotYTZ4ZHlaeURMcnRacE9Zc0J2TWt4VktTQWdFV3BlNXBzWmlfMXFEZFRiYWRIMmV3X3ItaWc0T3pzOG52THI4c1RQaDY1RWdNbXItTTUtdlFTS1d6SUpZTVlXM2lOTWtLWXF6TGNSRE9OWkJQSUs3UXFoSEtOa2NpNEJLeTFOektldFVUVHk4cFJCSE5Qdw?oc=5</t>
         </is>
       </c>
       <c r="I33" s="2" t="inlineStr"/>
@@ -1956,12 +1956,12 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Corporate Tax</t>
+          <t>VAT</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
@@ -1971,12 +1971,12 @@
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
-          <t>UAE tax warning as thousands of businesses approach Corporate Tax deadline - Arabian Business</t>
+          <t>Number of retail outlets connected to Digital Tourist VAT Refund System reaches more than 19,300 - Big News Network.com</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>News — UAE Corporate Tax</t>
+          <t>News — UAE VAT</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -1986,7 +1986,7 @@
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMidEFVX3lxTFBGbVZOWkkxM2FaVGlfeENJVWJXYzN6SDdmNk9nOFBYWWJDV3N6eGxVcnBRRXc5cDY5Qy1xSnNBQzVHMXR3NGpacEVucjlTMFRSaHc0dG5aZXc1aUVwSXlrTXhFTGd3RWNMbzVpWmdEVUZuUC1N?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi2AFBVV95cUxNUjRVVzdLOXJQTXpUZDhqeWlQNDAwVDV2ZmJqd3h4cW5ZbXc0cHEzZGJBSWlLOTk0ZlFFbXlVSThCUEtxcGFqUHYzSlRmeXF0bC1XQ1J3VVhKUUkzeVBfNTc4cmQwNmlRYldwUU01YXpmc0pxT0daNWRpRUwtM0N3MlBBR09rRldZZlA5bXVJOXVTcVZSeE5ldWRHSWhna0ZfTTNwZWEwODlFTXRRYnRhOVJVcHJ3dDRuSnZtQlBhc0NMa2dhSzk4b1lBWEx5Uk5Ld2RMaFdmNUY?oc=5</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr"/>
@@ -2001,12 +2001,12 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Corporate Tax</t>
+          <t>VAT</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
@@ -2016,12 +2016,12 @@
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>UAE reminds small businesses to file corporate tax returns even if no tax is due - Gulf News</t>
+          <t>UAE tourists can claim VAT refunds at 19,340 stores and on Noon purchases - Gulf News</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>News — UAE Corporate Tax</t>
+          <t>News — UAE VAT</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
@@ -2031,7 +2031,7 @@
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi0gFBVV95cUxOTm96UlB4Q2xPRlcybWNBanAtYXhxQkg0eHVCNDBvZlZGTWNGNzlSekNuVWZCU1JvOWR4MWxLanJMZEsyRms3NnZDSU90RnZuTkhad3pLLU1XX2VWV215T21HMTBmbVF1X0hmakhwM1BYZVNUQXZEV3A1UmR0QkZxVlJ1VDV5dGVMMFJFSGRxckpYVkVMMmFNMFBBdE9MZnlFSjJ3MDFXNzg2UXd0SUthQlZrd1Zjdy1JTVFkMEZlU0VKc3lzQW84VDBGLXFfVF93SnfSAeQBQVVfeXFMUEpicHFURTEyaDByTG44RGZUZ2R0MGJwRmdpV0hydzNTdkVYd0lFZzNITm9ueldCQ0JUZjZ3dW1TZ0xCSHM1S3c5eXExQlZac3V6bGd5Q1EzWFljOVRrZkJWRV9XcnFQWHdzRHQzWDRiUFhHaXlKMldlZHp5YW9zMHh2emxiX0R3MXdva2NFZ2JwcnVBZk52dEh2UEhvTW9FYzlJQ2xWdWZPQmpteFpaWnNUV0lpUTRiT0hNRXdHQVg1Q1VibWZqVWdocjBVVHJtVVFUbVFBdjJoRndFUS1aMTc5SEVh?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxQeDRPcDE4QjJaSFU3Qm1wRGVaWXl6cjY2c3YyVDF3TmtqN1RYMkh0WDdoSm56QmlXU21xSllRQWt4WHNFU09vUWZpTEd3dVVMb0UxNy0yZG1ucUF6aXhIZ2dWVXpkVjVqa2hHUGN3VHNZWEticFZMXzNfb2NzaVpwOFFkOVAtNDhBY0xjSUo3bkh0WUg2ZEJ4Q0JDU05Td0FTLWlUWXNfN2JKeGJsTEg3NGFDMzNwT21JZTFGT0V30gHQAUFVX3lxTE9wdElvSG52YzNWWUt6WGJaRkp0LXpmVHpQTFV4WHczVkQtOUhOMWpqRzd2UjgyQjNOSWdMT3QwM1luZzdtNWhXdU91R2lqS0FKcG1hUGExZ1QxWG1SSUo2cWZSWll0bjdpQ2pBOXFjTUMxcjJma0RraGlVbjNjajZRM0h4OVZfM0FUQXNERTQzQm1TS29QVjdiQzM2T19naktoTXhfQ1pvNmx4U2IxVkkxUWF5QmZ4QUxmMXB2bFVvR2RVWm10bjE2SlNaRzJ2VEU?oc=5</t>
         </is>
       </c>
       <c r="I35" s="2" t="inlineStr"/>
@@ -2046,7 +2046,7 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
@@ -2061,12 +2061,12 @@
       </c>
       <c r="E36" s="3" t="inlineStr">
         <is>
-          <t>Federal Tax Authority wins SAP Global Innovation Award - SAP News Center</t>
+          <t>Retail outlets linked to UAE's Digital Tourist VAT Refund System exceed 19,300 - Emirates 24|7</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>News — UAE Corporate Tax</t>
+          <t>News — UAE VAT</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
@@ -2076,7 +2076,7 @@
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxQYWE1ODFVeGZ2UEVVd0IyYXY0ckdPdFp4blEzcm9pZTZ5dm1MUDlocTNzNnd4dTh3cVhQb0o2aHJ2Y2VjTndrd2d6N2t1eW9OTzVtQ2JrcXVwN2NidFd2WUViQlRleTVQQXNpV2VvOVkyMFRINHhnNXpsUWdOcDhDUk1TbkpTajRkcUFGblBfWXhRZVU?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiugFBVV95cUxOcXRBMGsxX1Q5SkJXcEFwWnV3c0VVc19jUnRkWU5yMVlPelltaEhvOWNLcEJxYi1KUExWMVlmZE1FOExZYklsRHU4N3lQZGppMDRnYUFaRU1OWHdwaVpiWWowOENidVJjbDFPeTQyQklzOGM5bXhQbDJrRFg2TkR6bUplTzJNZzl2M3dJT2FEeHVTTVNtTml6UEdoZUFDcVRCZWFHMGg1ejZoSWI1UWFCLV9zREotcmF3V0HSAdQBQVVfeXFMT3Q0RFN0V3FRSlNWV20tMm5hY1N5VHBVWmxzdnZGVXIwZU92VTZVRDVUVkRZM0Q1U1ZNZzFRcFlEWTc2ckk0UjZhcEN4YmZIZndTd284ZDQ3Z2Z4OS1mVGFUX2RwRzgyMWViTjEyQ19wdUxucXEtZWtFRm5tOWpId1VYYlRmd1Rkc2tlb3Q3THR0THZxZWt3Q1ZyTGVvZ2hUUzZPeTBPSzlER3FXR0ZvUnJiWk5vdlpwYlYxdmZjZnNTVEQxM3hSY1pyTGV5Qkk2d2lrejQ?oc=5</t>
         </is>
       </c>
       <c r="I36" s="2" t="inlineStr"/>
@@ -2089,35 +2089,39 @@
           <t>2026-08-09</t>
         </is>
       </c>
-      <c r="B37" s="2" t="inlineStr"/>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>VAT</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>official</t>
+          <t>news</t>
         </is>
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t>Ministry of Finance Adopts “Aani” and “Jaywan” as New Payment Channels for Federal Service Fees and Fines</t>
+          <t>Indians, Russians, Turks top list of tourists claiming the most VAT refunds in UAE - khaleejtimes.com</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>Ministry of Finance — News</t>
+          <t>News — UAE VAT</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>mof.gov.ae</t>
+          <t>news.google.com</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>https://mof.gov.ae/en/news/ministry-of-finance-adopts-aani-and-jaywan-as-new-payment-channels-for-federal-service-fees-and-fines/</t>
+          <t>https://news.google.com/rss/articles/CBMiugFBVV95cUxPek9sY1dJUkpRblhiYnJDdDExOW1yREdXd1oyZ1Yxb0FnZlBYNTd3SUxGWnVMenlZVGlqRlIxLUszNk1Jd3BpcF9rVE9XLVF1OWdhY01fd0gteTJFRkVJLVREMjl4ZVRGZHJacUxJREpRN3UxdHFncGhITEQ0MnUzTkhKY2FSZnBnaFUzZDEyRnZOdG1hOWVFX2FLNG9Ca1lGekQzcllxd0FqTUhvTTRZM3MxcElQV0JaMWfSAcIBQVVfeXFMT2FPTEx4WGUzNUNhZWdBa1MzVU5GN1p3SkRwM0o5TWlqenhqVTNhR1Z0bThyN0laMS1tOUhfaG1qMmZpQi1pT3lTNEhKT2l3SklKZ1E3MXkyYVBrMnUwOTh1Y2RxSkFISUdlT1B6Qm1tTV9CUV9YM0xwcTJ2NzVmWUcxaFJ2YzhYeVBjZG1WSG9vcVc2N2tqRzNreHFwWVpaaUdncndzVEVLaE8zeHczU0Jvdl9FazU2NE1CNWZqQmZmekE?oc=5</t>
         </is>
       </c>
       <c r="I37" s="2" t="inlineStr"/>
@@ -2130,7 +2134,11 @@
           <t>2026-08-09</t>
         </is>
       </c>
-      <c r="B38" s="2" t="inlineStr"/>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
           <t>VAT</t>
@@ -2138,27 +2146,27 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>official</t>
+          <t>news</t>
         </is>
       </c>
       <c r="E38" s="3" t="inlineStr">
         <is>
-          <t>Ministry of Finance Announces Decision introduces a Minimum Excise Price for Liquids Used in Electronic Smoking Devices Effective 1 September 2026</t>
+          <t>Tourists can now claim VAT refunds at 19,300 retail outlets across the UAE - Gulf Business</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>Ministry of Finance — News</t>
+          <t>News — UAE VAT</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>mof.gov.ae</t>
+          <t>news.google.com</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>https://mof.gov.ae/en/news/ministry-of-finance-announces-decision-introduces-a-minimum-excise-price-for-liquids-used-in-electronic-smoking-devices-effective-1-september-2026/</t>
+          <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxQV2tyUkVhVzNVUlZ0QW9LdW5PWV9OTEVSN1FHU2c0Um9qbTRDNXFIdmZUaERGcDFPUkkyTVpzWXBQblJHb1VzVERybTh5WkIzcnRoRFo1ZVBicVRMQXpFZXB3VVJRQVZ6UDNNZDItT1RuTXcxYWxtSU1PaGlPNTFNUnpzLXBGX2QxSy1WVjU4alg4Q0dEWmY4WFZ6cEt1a1FZQXpRODFFN0xRT3VwSWFfNw?oc=5</t>
         </is>
       </c>
       <c r="I38" s="2" t="inlineStr"/>
@@ -2171,40 +2179,752 @@
           <t>2026-08-09</t>
         </is>
       </c>
-      <c r="B39" s="2" t="inlineStr"/>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>Corporate Tax</t>
+          <t>VAT</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>official</t>
+          <t>news</t>
         </is>
       </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
-          <t>Ministry of Finance Announces Extension of Small Business Relief for Corporate Tax Purposes until 31 December 2029</t>
+          <t>UAE tourists can now claim VAT refunds on eligible Noon online shopping purchases - Arabian Business</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>Ministry of Finance — News</t>
+          <t>News — UAE VAT</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>mof.gov.ae</t>
+          <t>news.google.com</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>https://mof.gov.ae/en/news/ministry-of-finance-announces-extension-of-small-business-relief-for-corporate-tax-purposes-until-31-december-2029/</t>
+          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxNSk0xOTlEQk5DQm4tczlCUE1jZ1dmamdsaUQ2TUYwWnlNd2JHMjhhVXZVUF8wNGpSVUFRNXhvU01pY01FMlUwWEt0anFyS3Q3QS0wa3BjZE1YLWtkWkpYeUJxVmlaSUhQM0Z3Mk9odUFYenhNRnBZeUkyQ0doNWJ2VGUySGY2dG9kMnlJaWhuWEMzb25aWjA1VXZkLWRwelk1MXJjbjBrV2F1Z29KZTJ3?oc=5</t>
         </is>
       </c>
       <c r="I39" s="2" t="inlineStr"/>
       <c r="J39" s="2" t="inlineStr"/>
       <c r="K39" s="2" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>VAT</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>news</t>
+        </is>
+      </c>
+      <c r="E40" s="3" t="inlineStr">
+        <is>
+          <t>FTA issues five binding VAT directives on tax transactions - kpmg.com</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>News — UAE VAT</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>news.google.com</t>
+        </is>
+      </c>
+      <c r="H40" s="2" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxQQXptRUZOQlpWYUZiNzd1QThPVDhlUGM3TF9PU3NKZjUyS2lucEZLUUFKZFpfZVhXLWxteTBKbU1OVEU1WXdPVlViT2ZBb2h5dmlHa0Z2bjd0SzMxa1p6TzF0ajhuVFVSaUpkczUxd1lzeGVCeDNwRnpPbXJVNVNGWHB4UTcwR2dCYTJoWTVSYkJGQmxRZE42cXNmOExtclgxR28tUUdYVFRzaE92?oc=5</t>
+        </is>
+      </c>
+      <c r="I40" s="2" t="inlineStr"/>
+      <c r="J40" s="2" t="inlineStr"/>
+      <c r="K40" s="2" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>Corporate Tax</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>news</t>
+        </is>
+      </c>
+      <c r="E41" s="3" t="inlineStr">
+        <is>
+          <t>UAE extends Corporate Tax Small Business Relief until end of 2029 - travelsdubai.com</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>News — UAE Corporate Tax</t>
+        </is>
+      </c>
+      <c r="G41" s="2" t="inlineStr">
+        <is>
+          <t>news.google.com</t>
+        </is>
+      </c>
+      <c r="H41" s="2" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMingFBVV95cUxOYzFrN28yN3RDREhxYV9CVHl3UGU1NlpvSFJqaHJGWVpraVhEOEtqTnZVQk1OTjVjX1djWENocHdtYy1WY1dBSHZncjg3aGxWOXlwcFktaVVxYzBmZllLbzBaLUUxSEpyNW1HX3V5MG9YMWhTcjNfcnZxQ1JKRHZkMjlYSjlmUHk1SGFEYy0tYmlqWE96ajBqUnNSS19TUQ?oc=5</t>
+        </is>
+      </c>
+      <c r="I41" s="2" t="inlineStr"/>
+      <c r="J41" s="2" t="inlineStr"/>
+      <c r="K41" s="2" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>VAT</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>news</t>
+        </is>
+      </c>
+      <c r="E42" s="3" t="inlineStr">
+        <is>
+          <t>UAE seizes 3.58 million non-compliant excise goods - Gulf News</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>News — UAE Corporate Tax</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>news.google.com</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipwFBVV95cUxOOF9vUDk3UXlsY19FUWtOOEJ2V3Awam9fY09zeS1seXpTUUt2Y05TQlVUVjlwYlVuX2hRN3JBM095eTlqZ3pxWWx5ZWJzUzV1bGdCQ21JMzd1bjRIMGRMdHpiZWVOM1lmOVdtSXlicW4wYUNoYjMySjFTNl9OTnRvYWZycGdhODlTcU9sQUpwUEdJcnltNF9nSXpBWkpJbjF0VG1qeVJqTdIBugFBVV95cUxPMDVISGFVMTVqWFFiS0VMTmlzZzlyWXRVUl9BTjBGaWgtS21lN05BdlppYlVNQkNtYmZWaHRIczNlSWRmbXBBdG9zamlobjFhTFh6R2lYZFJ1RUtKWGZqOWpNd21LTmNxaUF1SjVIUm9UNjF6cmwxUGY2ZHFIVHBFdVJNMXcyeFp3dUZ2V1hpVmtnRmZOY29nLWNWQmxsQ0tHUzd0RjRyRUlZeW1adThtZEpPVl9KT1pFRUE?oc=5</t>
+        </is>
+      </c>
+      <c r="I42" s="2" t="inlineStr"/>
+      <c r="J42" s="2" t="inlineStr"/>
+      <c r="K42" s="2" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>Corporate Tax</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>news</t>
+        </is>
+      </c>
+      <c r="E43" s="3" t="inlineStr">
+        <is>
+          <t>UAE Extends Small Business Relief for Corporate Tax to 2029 - tbreak.com</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>News — UAE Corporate Tax</t>
+        </is>
+      </c>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>news.google.com</t>
+        </is>
+      </c>
+      <c r="H43" s="2" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMifEFVX3lxTE9icS1QSXhYc09ROHVJdzRtdXJTMEdLa0o5Mm5TZ3VxR002a3lTeFR5anZqRmNtcVEyQWxfQ050UFVOZnFBcFdwT1VoNGlVZU9xYkY2WkM5SlpSSnp6QkpHck5rTUxqOXNjNjM0UmFTQkFfOXZySFFON1pCSXc?oc=5</t>
+        </is>
+      </c>
+      <c r="I43" s="2" t="inlineStr"/>
+      <c r="J43" s="2" t="inlineStr"/>
+      <c r="K43" s="2" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>Corporate Tax</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>news</t>
+        </is>
+      </c>
+      <c r="E44" s="3" t="inlineStr">
+        <is>
+          <t>UAE extends corporate tax relief for small businesses until end of 2029 - Gulf News</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>News — UAE Corporate Tax</t>
+        </is>
+      </c>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t>news.google.com</t>
+        </is>
+      </c>
+      <c r="H44" s="2" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMixgFBVV95cUxNNEo4Tm9qN1dERmwzZ0tMR0ZOSUVQTkpOTTNiTDc1U2VaSTkyRkExekRzRjUzb2xrelYzV0oydU1qS2JCbHJXd1hxeWhPdmtUN1UtcXRCOHZpSXBxMlBMdFRKbDNxYlNFaVdwRXROTUVxWC1tZUpObDVIZzNVUDEzSUZpNkIxN3ctTDRNWU9xOUx6QXZieFdVV1hkNHhlcldHUzY5b21BZ1J2VTVhMlN2a1V5V1dJRkw1OTItdWo5Qzk5N2lPX1HSAdgBQVVfeXFMTmRQM08wYWhkelVySDhudHZWLWQyZ2lyUG9TNEJhWVV6ejAybDV6QXdvUFR5ZndxZldxWHVDMjRKVm1Ndm0yeE1HZHo1LXoyVFBzMkhuUDZESEw5RUFIaWlfNEdObjNxRlc4VFpOZVQ3RDhhellsdEpYN3pLVzl1d1Fva3R0RWpDb0d5cVN0Z3I3emowS2tNbkplWTh1Z2NvVkRMd0R3STNWV3hrUVFtd3hxdjQxWjI2ZU4wVE9JTzlsWVUwYXlPTmU4YWJmazMxQk93MHVHbGZE?oc=5</t>
+        </is>
+      </c>
+      <c r="I44" s="2" t="inlineStr"/>
+      <c r="J44" s="2" t="inlineStr"/>
+      <c r="K44" s="2" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>Corporate Tax</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>news</t>
+        </is>
+      </c>
+      <c r="E45" s="3" t="inlineStr">
+        <is>
+          <t>Small businesses in UAE urged to file corporate tax returns before deadline, says FTA - khaleejtimes.com</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>News — UAE Corporate Tax</t>
+        </is>
+      </c>
+      <c r="G45" s="2" t="inlineStr">
+        <is>
+          <t>news.google.com</t>
+        </is>
+      </c>
+      <c r="H45" s="2" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxOWnJlYmRmRm4xdy0xZ0toMUNUbnhTd3A5UW1pVzhFeXhIM2txamo4NU5qYVYwZGlQcEYwLTJhelBkOEdHajRYSE5PRnZtdmxGWmc0R2JlUVk0eVc0aW53NzdlM08zeWFzTUNocU9UcnY3UTNhTHVzZHhjRXFPZ0ZMMHMyRExEcjFiVVhKVzMxYk9FSHUxdERQRnUyZlJLWXA0ZVHSAaoBQVVfeXFMT3BwVV9lZzBQRTFjWUNVNEFzaUlhOUJuTHByVVRhdjRTbjdpajdOTjRtc2hfOEotMWlSb0FvX1F3azI2czNjMHREWnRJbFptM0F5ZHJkWUFsMW5fMDBsNU1YODgzT2VkMWZacU51MzkxaHJ0S216TF9UR241SnM0OVo2eHlDM0F6V2VfbUt4elZfZVBub2pLNW5fazhqV1hNUnBzRmkxS0NUQVE?oc=5</t>
+        </is>
+      </c>
+      <c r="I45" s="2" t="inlineStr"/>
+      <c r="J45" s="2" t="inlineStr"/>
+      <c r="K45" s="2" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>Corporate Tax</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>news</t>
+        </is>
+      </c>
+      <c r="E46" s="3" t="inlineStr">
+        <is>
+          <t>UAE extends Corporate Tax relief until 2029 for businesses earning up to $817,000 - Arabian Business</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>News — UAE Corporate Tax</t>
+        </is>
+      </c>
+      <c r="G46" s="2" t="inlineStr">
+        <is>
+          <t>news.google.com</t>
+        </is>
+      </c>
+      <c r="H46" s="2" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMieEFVX3lxTE5SM3FoRTVUSmJwTlpLbi1vOGFPM3RPcXpraXlCUG9iQlhuUUJ2MGRCczd6aDM0MFFNWS0yS2tNNVIxYjd2Y3AxWExhUnJNcHNXT3dLdGhyV2FBQUQwbmZ3YjRZc3NXTkNoLU5HTFRkTWRkSlZ6TEtHbg?oc=5</t>
+        </is>
+      </c>
+      <c r="I46" s="2" t="inlineStr"/>
+      <c r="J46" s="2" t="inlineStr"/>
+      <c r="K46" s="2" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>Corporate Tax</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>news</t>
+        </is>
+      </c>
+      <c r="E47" s="3" t="inlineStr">
+        <is>
+          <t>Ministry of Finance announces extension of small business relief for corporate tax purposes until 31 December 2029 - Zawya</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>News — UAE Corporate Tax</t>
+        </is>
+      </c>
+      <c r="G47" s="2" t="inlineStr">
+        <is>
+          <t>news.google.com</t>
+        </is>
+      </c>
+      <c r="H47" s="2" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMihwJBVV95cUxOWVAwdTI2R09XSWRHaFNWYkNGdUJsSTNnaGpRandNeklubW8zM2h3VkNIcmRiQTVrZUxlSnhydWtqUGVTRS1vYVVQWWJfY2swUzhYOFJrdHVCQTlvTk1LNVBfWjBPbHZxWVU5Q0xQVWFHbTlLYlE0ek1aWFhqaUF3dDlTY2p2T0dtV3gzSXhaWkdFdWFBejA5ZkhDSkVPanZUWDk0d1oxNlJOUkNxMER2M1oyc3Nla2NnUW9WYmFRS04zeGlCcjQ1YVNZT2ZraU5EN0h2ZWRDaklZTjFQUklLWmRGRVFkUjhKUjBybHA5UktLZHFiVnUtOFpuNmhSZ0o3YVV3eld3WQ?oc=5</t>
+        </is>
+      </c>
+      <c r="I47" s="2" t="inlineStr"/>
+      <c r="J47" s="2" t="inlineStr"/>
+      <c r="K47" s="2" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>Corporate Tax</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>news</t>
+        </is>
+      </c>
+      <c r="E48" s="3" t="inlineStr">
+        <is>
+          <t>FTA reminds small businesses to file corporate tax returns - Sharjah24</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>News — UAE Corporate Tax</t>
+        </is>
+      </c>
+      <c r="G48" s="2" t="inlineStr">
+        <is>
+          <t>news.google.com</t>
+        </is>
+      </c>
+      <c r="H48" s="2" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiW0FVX3lxTE5NZ1VTdFlkVERkd0pETmFiVUQzZzEySVNaeWFyV2N3MHdhSWZreEZnUDFCYXhiWGtCOVVxMFdWUzhDa3JCU1czenE3QzJzaG0tNU5iMkFmRFRsTUU?oc=5</t>
+        </is>
+      </c>
+      <c r="I48" s="2" t="inlineStr"/>
+      <c r="J48" s="2" t="inlineStr"/>
+      <c r="K48" s="2" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>Corporate Tax</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>news</t>
+        </is>
+      </c>
+      <c r="E49" s="3" t="inlineStr">
+        <is>
+          <t>UAE extends small business relief for corporate tax until December 2029 - TradeArabia</t>
+        </is>
+      </c>
+      <c r="F49" s="2" t="inlineStr">
+        <is>
+          <t>News — UAE Corporate Tax</t>
+        </is>
+      </c>
+      <c r="G49" s="2" t="inlineStr">
+        <is>
+          <t>news.google.com</t>
+        </is>
+      </c>
+      <c r="H49" s="2" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxOc3RJWW11LUNyUERIeHh0dTVRVFJySzBoWVB0N1RCdVNpTVpORW03RkVXaG1pdk5HbWJfTDUzYXRIellIdlo4dVBXcXpuZHNrQXZRMk5MMGF1UkpqbGRTbXZRekZTYkU3cHpsdmJHdTVRdFFxSE1aSzZxWW1rb0RuT1RNZzVOWG91OGVTcFZVUGFVLWRUY3JsRnEtYkR4WUJjWnp6NkljSUd2NExsdUYtVA?oc=5</t>
+        </is>
+      </c>
+      <c r="I49" s="2" t="inlineStr"/>
+      <c r="J49" s="2" t="inlineStr"/>
+      <c r="K49" s="2" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>Corporate Tax</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>news</t>
+        </is>
+      </c>
+      <c r="E50" s="3" t="inlineStr">
+        <is>
+          <t>UAE tax warning as thousands of businesses approach Corporate Tax deadline - Arabian Business</t>
+        </is>
+      </c>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>News — UAE Corporate Tax</t>
+        </is>
+      </c>
+      <c r="G50" s="2" t="inlineStr">
+        <is>
+          <t>news.google.com</t>
+        </is>
+      </c>
+      <c r="H50" s="2" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMidEFVX3lxTFBGbVZOWkkxM2FaVGlfeENJVWJXYzN6SDdmNk9nOFBYWWJDV3N6eGxVcnBRRXc5cDY5Qy1xSnNBQzVHMXR3NGpacEVucjlTMFRSaHc0dG5aZXc1aUVwSXlrTXhFTGd3RWNMbzVpWmdEVUZuUC1N?oc=5</t>
+        </is>
+      </c>
+      <c r="I50" s="2" t="inlineStr"/>
+      <c r="J50" s="2" t="inlineStr"/>
+      <c r="K50" s="2" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>Corporate Tax</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>news</t>
+        </is>
+      </c>
+      <c r="E51" s="3" t="inlineStr">
+        <is>
+          <t>UAE reminds small businesses to file corporate tax returns even if no tax is due - Gulf News</t>
+        </is>
+      </c>
+      <c r="F51" s="2" t="inlineStr">
+        <is>
+          <t>News — UAE Corporate Tax</t>
+        </is>
+      </c>
+      <c r="G51" s="2" t="inlineStr">
+        <is>
+          <t>news.google.com</t>
+        </is>
+      </c>
+      <c r="H51" s="2" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi0gFBVV95cUxOTm96UlB4Q2xPRlcybWNBanAtYXhxQkg0eHVCNDBvZlZGTWNGNzlSekNuVWZCU1JvOWR4MWxLanJMZEsyRms3NnZDSU90RnZuTkhad3pLLU1XX2VWV215T21HMTBmbVF1X0hmakhwM1BYZVNUQXZEV3A1UmR0QkZxVlJ1VDV5dGVMMFJFSGRxckpYVkVMMmFNMFBBdE9MZnlFSjJ3MDFXNzg2UXd0SUthQlZrd1Zjdy1JTVFkMEZlU0VKc3lzQW84VDBGLXFfVF93SnfSAeQBQVVfeXFMUEpicHFURTEyaDByTG44RGZUZ2R0MGJwRmdpV0hydzNTdkVYd0lFZzNITm9ueldCQ0JUZjZ3dW1TZ0xCSHM1S3c5eXExQlZac3V6bGd5Q1EzWFljOVRrZkJWRV9XcnFQWHdzRHQzWDRiUFhHaXlKMldlZHp5YW9zMHh2emxiX0R3MXdva2NFZ2JwcnVBZk52dEh2UEhvTW9FYzlJQ2xWdWZPQmpteFpaWnNUV0lpUTRiT0hNRXdHQVg1Q1VibWZqVWdocjBVVHJtVVFUbVFBdjJoRndFUS1aMTc5SEVh?oc=5</t>
+        </is>
+      </c>
+      <c r="I51" s="2" t="inlineStr"/>
+      <c r="J51" s="2" t="inlineStr"/>
+      <c r="K51" s="2" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>VAT</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>news</t>
+        </is>
+      </c>
+      <c r="E52" s="3" t="inlineStr">
+        <is>
+          <t>Federal Tax Authority wins SAP Global Innovation Award - SAP News Center</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t>News — UAE Corporate Tax</t>
+        </is>
+      </c>
+      <c r="G52" s="2" t="inlineStr">
+        <is>
+          <t>news.google.com</t>
+        </is>
+      </c>
+      <c r="H52" s="2" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxQYWE1ODFVeGZ2UEVVd0IyYXY0ckdPdFp4blEzcm9pZTZ5dm1MUDlocTNzNnd4dTh3cVhQb0o2aHJ2Y2VjTndrd2d6N2t1eW9OTzVtQ2JrcXVwN2NidFd2WUViQlRleTVQQXNpV2VvOVkyMFRINHhnNXpsUWdOcDhDUk1TbkpTajRkcUFGblBfWXhRZVU?oc=5</t>
+        </is>
+      </c>
+      <c r="I52" s="2" t="inlineStr"/>
+      <c r="J52" s="2" t="inlineStr"/>
+      <c r="K52" s="2" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="inlineStr"/>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>official</t>
+        </is>
+      </c>
+      <c r="E53" s="3" t="inlineStr">
+        <is>
+          <t>Ministry of Finance Adopts “Aani” and “Jaywan” as New Payment Channels for Federal Service Fees and Fines</t>
+        </is>
+      </c>
+      <c r="F53" s="2" t="inlineStr">
+        <is>
+          <t>Ministry of Finance — News</t>
+        </is>
+      </c>
+      <c r="G53" s="2" t="inlineStr">
+        <is>
+          <t>mof.gov.ae</t>
+        </is>
+      </c>
+      <c r="H53" s="2" t="inlineStr">
+        <is>
+          <t>https://mof.gov.ae/en/news/ministry-of-finance-adopts-aani-and-jaywan-as-new-payment-channels-for-federal-service-fees-and-fines/</t>
+        </is>
+      </c>
+      <c r="I53" s="2" t="inlineStr"/>
+      <c r="J53" s="2" t="inlineStr"/>
+      <c r="K53" s="2" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr"/>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>VAT</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>official</t>
+        </is>
+      </c>
+      <c r="E54" s="3" t="inlineStr">
+        <is>
+          <t>Ministry of Finance Announces Decision introduces a Minimum Excise Price for Liquids Used in Electronic Smoking Devices Effective 1 September 2026</t>
+        </is>
+      </c>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>Ministry of Finance — News</t>
+        </is>
+      </c>
+      <c r="G54" s="2" t="inlineStr">
+        <is>
+          <t>mof.gov.ae</t>
+        </is>
+      </c>
+      <c r="H54" s="2" t="inlineStr">
+        <is>
+          <t>https://mof.gov.ae/en/news/ministry-of-finance-announces-decision-introduces-a-minimum-excise-price-for-liquids-used-in-electronic-smoking-devices-effective-1-september-2026/</t>
+        </is>
+      </c>
+      <c r="I54" s="2" t="inlineStr"/>
+      <c r="J54" s="2" t="inlineStr"/>
+      <c r="K54" s="2" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr"/>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>Corporate Tax</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>official</t>
+        </is>
+      </c>
+      <c r="E55" s="3" t="inlineStr">
+        <is>
+          <t>Ministry of Finance Announces Extension of Small Business Relief for Corporate Tax Purposes until 31 December 2029</t>
+        </is>
+      </c>
+      <c r="F55" s="2" t="inlineStr">
+        <is>
+          <t>Ministry of Finance — News</t>
+        </is>
+      </c>
+      <c r="G55" s="2" t="inlineStr">
+        <is>
+          <t>mof.gov.ae</t>
+        </is>
+      </c>
+      <c r="H55" s="2" t="inlineStr">
+        <is>
+          <t>https://mof.gov.ae/en/news/ministry-of-finance-announces-extension-of-small-business-relief-for-corporate-tax-purposes-until-31-december-2029/</t>
+        </is>
+      </c>
+      <c r="I55" s="2" t="inlineStr"/>
+      <c r="J55" s="2" t="inlineStr"/>
+      <c r="K55" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update: 2026-08-12 04:40 UTC
</commit_message>
<xml_diff>
--- a/docs/tax_updates_export.xlsx
+++ b/docs/tax_updates_export.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K55"/>
+  <dimension ref="A1:K59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -511,32 +511,32 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Transfer Pricing</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>commentary</t>
+          <t>news</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>Tax Insights: Canada introduces a simplified transfer pricing documentation regime - PwC</t>
+          <t>Foreign outflows in July were the lowest in the GCC - EnterpriseAM</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>News — Big 4 UAE Tax Commentary</t>
+          <t>News — UAE E-Invoicing</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -546,7 +546,7 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiwAFBVV95cUxOVm8yXzZQUVY4R2djbXBUdHQ0aFUyQnFaSHNxSkFCbTNxNmxSVTZVUHRxa1lvVnF2Nlk2bmhTQ2w4ejJaTVR2NUY4S3VsajBFTEV2dkRwbk9BbEh1MWtwczNVNHgtQm1yaFJwc2NlZldqM053NGhwbE1TLWR3eDNIQ3V2ZzhTQ2JmbVJlNlliMkRoalBfYzQ3WHdVaXR2R2MzNEw1dGRQNzFfRWxTWklzYkJNYVZKVjFMclFQQjIzMUU?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiW0FVX3lxTE8tRko4Unh0QWI1ekpUTHJ3QmktT1dyWXd2S2REcHZIZVVvd2Rtdm1WSkUtQUtacjlnSGlLdWtIMk0tVVNxU1ZKTU1qSVdpc2NOUjBGWUh5STBrM0E?oc=5</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr"/>
@@ -556,12 +556,12 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -571,17 +571,17 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>commentary</t>
+          <t>news</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>Canada launches public consultations on steel imports and imposes surtax on wood cabinets and vanities - EY</t>
+          <t>UAE extends small business tax relief until 2029 - Yahoo Finance</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>News — Big 4 UAE Tax Commentary</t>
+          <t>News — UAE E-Invoicing</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -591,7 +591,7 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMigAFBVV95cUxNMy1qdEVRaXhDVUZ4c3FTNUlCS0F0SEhoRnQtRk5BTnB1d2VFSmZSUk95RmRSdEw4LUFBV1FwYTIwbTVLZHdqOEdkcDhRb29fWDc1cGN0ZFA3a0habW9iY0NWam9LZmtfa3c2NDlLZ3N1MVJYWWRwejlhM1ViSndzZg?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMimwFBVV95cUxNM2FhblZZVW5LVzI2bmRYWFhadXJ5bGU2OU54U3UzTmpGWmlweXlYTVVSWHpXaXU5YnJLNlh0STNsNmhYdG9feTdsN2xKNWlNSGZRM3loRllITXB4U0ljUkpyYllpLU9jQUZVOVdab1Rocml1OWxsa1lKWE00Wk42QWZRejVCaTk4QllWdTJTMWxJd2RKbVZiWHo4UQ?oc=5</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr"/>
@@ -601,17 +601,17 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
           <t>2026-08-11</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-07</t>
-        </is>
-      </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Corporate Tax</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -621,12 +621,12 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>UAE extends Small Business Relief for corporate tax - Absolute Geeks</t>
+          <t>UAE seizes 8.45m non-compliant tobacco and drink products in six-month tax drive - Gulf News</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>News — FTA Announcements</t>
+          <t>News — UAE VAT</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -636,7 +636,7 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxPWU10OExoZmlXRjdCamp5VHROMnNDb1dKN1I3NE85dTI4aU84VjVvczlyanRyWEw4OVBuOWpVa1NJZm9qQ2hSZl9YYlhxOGNEYXBCeDlGQVF1RUV1TWJlSGVmdnpHRktyS2ktV2IwQ0s3T3hZMzV4Ni03aGdvVTNHZFhEYThmRE5uclJqR1BKUF90MXktS2xEaXctR0RsLXphM0g0REdvWHY?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiygFBVV95cUxOeXEwYUYyRVl3dzRiREtKU01zOTFJNXZCNVpNcE5wYTUxRUN3U1A0SkxudUUxYkI0WHUzUmZoelZBLUJSaUFFcno2WFc5bzNBR2FQZU4zSkFuMTNWbkcyMVNMdXc3dmplcVNLdDRsN2xDdng3ZFg2UnFiREgzZHIwUFlpUkhxdXdkeG0ySXJQS2Q2LWJJRGxrbWZMT3AxTU9KWWM1OS1qQ2FET0oyQjhhZFNXX3RDWklhU3VrdTM2aTRRcFIxdXlWOHJB0gHcAUFVX3lxTFA5OFBJbzlhcVVXbXNwNWtBamtpbFdwbVkxdHFtSTJXWk9TR3kxZ0F6UFVtQy1EYnpaZUM2Vmp1enVjeFJoSjR1ekpMenVHdEhaTlhGdmxKUzQwV1BsQnpiNXg0UDRpTndaTjE2RTJBNzFIbzNEZExXWlhmVnpYT2VTbmFsNldOZVlzX3BsaU5xUUplai13SEl2RUdpNG0tWTJOd1BCQkVaUVowX0NiZHF3VU1BLU5VcVpBb2RoRXVERGdaYmxhMmhEd3MxNVRoekNKQ3hZeEhyWkUwQUg?oc=5</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr"/>
@@ -646,17 +646,17 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
           <t>2026-08-11</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-04</t>
-        </is>
-      </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Corporate Tax</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -666,12 +666,12 @@
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>Spotify forecasts slower growth despite AI investment - Gulf Business</t>
+          <t>UAE Extends Small Business Relief for Corporate Tax Purposes Until 2029 - entARABI</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>News — FTA Announcements</t>
+          <t>News — UAE Corporate Tax</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -681,7 +681,7 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMilwFBVV95cUxNQUhDU0xPaGxHNTZZdDNmRFRsTndvQThIUkRVV0hyTkpVbWhFNXdsZ2hjUXFrNzByWEc1ZUdITm1FYkM2N3k5MW5paDBud1RfNGF4MXNIdlluaVktTVRfd0RlZzJpUmc0UlZ2WUlKU1VDTUdELXpoelU0Z2kteENFZjVfcWx5YmhLc21jS3J5VXVkeEZ3UXRV?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMipwFBVV95cUxOV0NzYjBEMHBFM0dLeTRxdURMWjYtZUZ2OXpSTENyYVozcGpPWkVBb09JaU1pQjAtWEVTdlcyQ1VjbmNGc2NiT05jWFUxMTNFVzFJMHlHQlY3VmxDaU9XUVZwY21yS1ZFYldWckFZallwVDU3Y1ZzLVNKbndvMXVGckJFMnRWNUtNOTFzRlgzUDhMbHFpMEZsRk9XejN4S3F4cld0aTJPdw?oc=5</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr"/>
@@ -696,27 +696,27 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>VAT</t>
+          <t>Transfer Pricing</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>news</t>
+          <t>commentary</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>UAE Sets Minimum Excise Price for E-Liquids - Vaping360</t>
+          <t>Tax Insights: Canada introduces a simplified transfer pricing documentation regime - PwC</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>News — FTA Announcements</t>
+          <t>News — Big 4 UAE Tax Commentary</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -726,7 +726,7 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMidkFVX3lxTE9HS2ZoOFFrdlRtX3N4ZXM5UlpzLTFKc21Pdi1CVkhNYW1PNGozMDBVYVZ0VjlrUDNCMFRQRG1hOGpPNllSd0dpX0dhNm02a3drdmZneHpQOUhtUkxXWlFBcDlETkt0dF9xalFRMldrVWZMSXh5NHc?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiwAFBVV95cUxOVm8yXzZQUVY4R2djbXBUdHQ0aFUyQnFaSHNxSkFCbTNxNmxSVTZVUHRxa1lvVnF2Nlk2bmhTQ2w4ejJaTVR2NUY4S3VsajBFTEV2dkRwbk9BbEh1MWtwczNVNHgtQm1yaFJwc2NlZldqM053NGhwbE1TLWR3eDNIQ3V2ZzhTQ2JmbVJlNlliMkRoalBfYzQ3WHdVaXR2R2MzNEw1dGRQNzFfRWxTWklzYkJNYVZKVjFMclFQQjIzMUU?oc=5</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr"/>
@@ -741,27 +741,27 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>E-Invoicing</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>news</t>
+          <t>commentary</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>E-Invoicing Readiness Checklist: How UAE Businesses Can Prepare Before the Deadline - NewsBreak: Local News &amp; Alerts</t>
+          <t>Canada launches public consultations on steel imports and imposes surtax on wood cabinets and vanities - EY</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>News — UAE E-Invoicing</t>
+          <t>News — Big 4 UAE Tax Commentary</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -771,7 +771,7 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMixgFBVV95cUxPQmFubHpKbnIzS2N1cVJkbFA5bDRWcUhzQ0lYazZ3Z0ZBazZKQzVoTjRxZXBrMFNNSGNXTGp4ZG1EZ0xTTGFwanZQZkxvbjA5UFQxYkNBLWF6bEtDSlB5UlcyNU9fc2E1VTRNMWtTYnRyOFRlTUxjRlVlcEVwRVdDb05OQlo4VC1GcUpqUkpmVzhsUmc0RGJrZlJWN0tCMXVQc0d5dTEtT055TFRDT3c5R2pUN1hpaEF3R21TOHo2d1pNZldNcUE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMigAFBVV95cUxNMy1qdEVRaXhDVUZ4c3FTNUlCS0F0SEhoRnQtRk5BTnB1d2VFSmZSUk95RmRSdEw4LUFBV1FwYTIwbTVLZHdqOEdkcDhRb29fWDc1cGN0ZFA3a0habW9iY0NWam9LZmtfa3c2NDlLZ3N1MVJYWWRwejlhM1ViSndzZg?oc=5</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr"/>
@@ -786,12 +786,12 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Corporate Tax</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -801,12 +801,12 @@
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>A jumpy July - EnterpriseAM</t>
+          <t>UAE extends Small Business Relief for corporate tax - Absolute Geeks</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>News — UAE E-Invoicing</t>
+          <t>News — FTA Announcements</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -816,7 +816,7 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiXkFVX3lxTFBCcFdtSjE1bW5pMlREMHVqWTYwcW1xajViLWZvTmU1MUk0MUZiX2pPay12Nm5RS0tzdmJjYU9VY2hjUi10enNsYk1qcEZqc3FQc3dEZE1CaTJRYTJvVWc?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiqAFBVV95cUxPWU10OExoZmlXRjdCamp5VHROMnNDb1dKN1I3NE85dTI4aU84VjVvczlyanRyWEw4OVBuOWpVa1NJZm9qQ2hSZl9YYlhxOGNEYXBCeDlGQVF1RUV1TWJlSGVmdnpHRktyS2ktV2IwQ0s3T3hZMzV4Ni03aGdvVTNHZFhEYThmRE5uclJqR1BKUF90MXktS2xEaXctR0RsLXphM0g0REdvWHY?oc=5</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr"/>
@@ -831,7 +831,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -846,12 +846,12 @@
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>Another Hormuz workaround - EnterpriseAM</t>
+          <t>Spotify forecasts slower growth despite AI investment - Gulf Business</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>News — UAE E-Invoicing</t>
+          <t>News — FTA Announcements</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -861,7 +861,7 @@
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMib0FVX3lxTE5iUjRXRTlrdVBXOHUyRWlYc2ttOXdYaVktOE5ZU1YxMnRLcnlHeWRPdl9CQmRkR3Bqc21aeFlWMmdFcGdjanc3d2RNTnRGcWdKVGdxQTZmeC02clJoSXJJaGJlUUM5TW5pQjRORkVpRQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMilwFBVV95cUxNQUhDU0xPaGxHNTZZdDNmRFRsTndvQThIUkRVV0hyTkpVbWhFNXdsZ2hjUXFrNzByWEc1ZUdITm1FYkM2N3k5MW5paDBud1RfNGF4MXNIdlluaVktTVRfd0RlZzJpUmc0UlZ2WUlKU1VDTUdELXpoelU0Z2kteENFZjVfcWx5YmhLc21jS3J5VXVkeEZ3UXRV?oc=5</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr"/>
@@ -876,12 +876,12 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>E-Invoicing</t>
+          <t>VAT</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -891,12 +891,12 @@
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>UAE e-invoicing: How digital invoices will transform business - Khaleej Times</t>
+          <t>UAE Sets Minimum Excise Price for E-Liquids - Vaping360</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>News — UAE E-Invoicing</t>
+          <t>News — FTA Announcements</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -906,7 +906,7 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMivwFBVV95cUxQMjFwZTd6MkpqcXZKaEwxZV9fUlZWSEtSeVdIQXN6YXFPMURFMWZhOHc0NWFuWlRfd1ZNX2doQVBpbXBqRFBTOVNNcjVTYVpOcEozYmtoaWxDUHVoUFFNT1RBWEI3RzJybmFWejFNcEcxYXpybDBiUzRLUk85ajBkOHIydnBjOUV6NEVJUjZkQTNOQ0Fud1BjdGtUNVpwTmlTazdyNWZmaXRwTkthY1Nac1RPWU90T3lMemJJNHp5VdIBvwFBVV95cUxQMjFwZTd6MkpqcXZKaEwxZV9fUlZWSEtSeVdIQXN6YXFPMURFMWZhOHc0NWFuWlRfd1ZNX2doQVBpbXBqRFBTOVNNcjVTYVpOcEozYmtoaWxDUHVoUFFNT1RBWEI3RzJybmFWejFNcEcxYXpybDBiUzRLUk85ajBkOHIydnBjOUV6NEVJUjZkQTNOQ0Fud1BjdGtUNVpwTmlTazdyNWZmaXRwTkthY1Nac1RPWU90T3lMemJJNHp5VQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMidkFVX3lxTE9HS2ZoOFFrdlRtX3N4ZXM5UlpzLTFKc21Pdi1CVkhNYW1PNGozMDBVYVZ0VjlrUDNCMFRQRG1hOGpPNllSd0dpX0dhNm02a3drdmZneHpQOUhtUkxXWlFBcDlETkt0dF9xalFRMldrVWZMSXh5NHc?oc=5</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr"/>
@@ -921,12 +921,12 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>E-Invoicing</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -936,7 +936,7 @@
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>More investments in Adnoc’s fleet, Indian IPOs, and Egypt’s North Coast - EnterpriseAM</t>
+          <t>E-Invoicing Readiness Checklist: How UAE Businesses Can Prepare Before the Deadline - NewsBreak: Local News &amp; Alerts</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
@@ -951,7 +951,7 @@
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiW0FVX3lxTE1RdV9pa3ZIMmpRWnFlcXRaeTRnSy1zZUp0enVScm1nc0hMX3UwTEdEOG9oQy00UUJiSUR4WENleElGQVVmLXh3ZE10b09nQWphT0IzNHNJb0h3Q0E?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMixgFBVV95cUxPQmFubHpKbnIzS2N1cVJkbFA5bDRWcUhzQ0lYazZ3Z0ZBazZKQzVoTjRxZXBrMFNNSGNXTGp4ZG1EZ0xTTGFwanZQZkxvbjA5UFQxYkNBLWF6bEtDSlB5UlcyNU9fc2E1VTRNMWtTYnRyOFRlTUxjRlVlcEVwRVdDb05OQlo4VC1GcUpqUkpmVzhsUmc0RGJrZlJWN0tCMXVQc0d5dTEtT055TFRDT3c5R2pUN1hpaEF3R21TOHo2d1pNZldNcUE?oc=5</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr"/>
@@ -966,7 +966,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -981,12 +981,12 @@
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>FTA Directive No. 5 of 2026 - Crowe</t>
+          <t>A jumpy July - EnterpriseAM</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>News — UAE VAT</t>
+          <t>News — UAE E-Invoicing</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -996,7 +996,7 @@
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiVkFVX3lxTE40S0RnRzF2d1dBSmNHdkNNQXZQQmlOYWNOSk5OWnlVNUN3ZDB5UHBUV29RXzNvaF9pVFNQZ2FwTUdocGhxMXp1T3gxMUFycGNESFA1bXNR?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiXkFVX3lxTFBCcFdtSjE1bW5pMlREMHVqWTYwcW1xajViLWZvTmU1MUk0MUZiX2pPay12Nm5RS0tzdmJjYU9VY2hjUi10enNsYk1qcEZqc3FQc3dEZE1CaTJRYTJvVWc?oc=5</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr"/>
@@ -1016,7 +1016,7 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>VAT</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
@@ -1026,12 +1026,12 @@
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>Digital currency and VAT: New UAE rules for businesses to consider - thenationalnews.com</t>
+          <t>Another Hormuz workaround - EnterpriseAM</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>News — UAE VAT</t>
+          <t>News — UAE E-Invoicing</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -1041,7 +1041,7 @@
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiugFBVV95cUxQamI1MElzOEtNS1ZjVWR3VGpjZjNUZjBXbjQwZkJIZ3AwOFVqckl0WWFQN2JpaEg5XzRTUTBVMDFOeVhMaUZxYW9GUnBFNW55WnhKd2ZKOVZoekRBWUNqQkp3dGFPZ2JQcWY5SjVlRUJuTURfcVN5aUNXVmthdUh4cHlJbFNHN3lyT1VTU2l2Nk92U09JZFh3eXp0c29jTlJNZW1VLTZBR2h5WmdBTjFuNGczZkZwdDY1QWc?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMib0FVX3lxTE5iUjRXRTlrdVBXOHUyRWlYc2ttOXdYaVktOE5ZU1YxMnRLcnlHeWRPdl9CQmRkR3Bqc21aeFlWMmdFcGdjanc3d2RNTnRGcWdKVGdxQTZmeC02clJoSXJJaGJlUUM5TW5pQjRORkVpRQ?oc=5</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr"/>
@@ -1056,12 +1056,12 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>E-Invoicing</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -1071,12 +1071,12 @@
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>Air India turbulence injures passengers on Phuket-Delhi flight - Gulf Business</t>
+          <t>UAE e-invoicing: How digital invoices will transform business - Khaleej Times</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>News — UAE Corporate Tax</t>
+          <t>News — UAE E-Invoicing</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -1086,7 +1086,7 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxOUk92b3hCQVZybGNndXNJOF9ZX0Z3TGl5NnRuXzE5NlBRb3czZXM2SkxXb3ZQSGNOdGo2a2U2b040ZVFDcFBqbzdvaFFZaVdBbFgwQkJOOEhDNzF6VXY1OU9Ca2t2Z1ZnQlhscXNXTVhDaWY3b2lvMUlEWFhkXzVxaDR3b191OUx2aTVKcEttYkFGTjRzRVpnbFJvLUZhYmNLTFJJNg?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMivwFBVV95cUxQMjFwZTd6MkpqcXZKaEwxZV9fUlZWSEtSeVdIQXN6YXFPMURFMWZhOHc0NWFuWlRfd1ZNX2doQVBpbXBqRFBTOVNNcjVTYVpOcEozYmtoaWxDUHVoUFFNT1RBWEI3RzJybmFWejFNcEcxYXpybDBiUzRLUk85ajBkOHIydnBjOUV6NEVJUjZkQTNOQ0Fud1BjdGtUNVpwTmlTazdyNWZmaXRwTkthY1Nac1RPWU90T3lMemJJNHp5VdIBvwFBVV95cUxQMjFwZTd6MkpqcXZKaEwxZV9fUlZWSEtSeVdIQXN6YXFPMURFMWZhOHc0NWFuWlRfd1ZNX2doQVBpbXBqRFBTOVNNcjVTYVpOcEozYmtoaWxDUHVoUFFNT1RBWEI3RzJybmFWejFNcEcxYXpybDBiUzRLUk85ajBkOHIydnBjOUV6NEVJUjZkQTNOQ0Fud1BjdGtUNVpwTmlTazdyNWZmaXRwTkthY1Nac1RPWU90T3lMemJJNHp5VQ?oc=5</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr"/>
@@ -1101,12 +1101,12 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Corporate Tax</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
@@ -1116,12 +1116,12 @@
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>UAE Business: UAE extends small business relief for corporate tax until December 2029 - Gulf Daily News</t>
+          <t>More investments in Adnoc’s fleet, Indian IPOs, and Egypt’s North Coast - EnterpriseAM</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>News — UAE Corporate Tax</t>
+          <t>News — UAE E-Invoicing</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -1131,7 +1131,7 @@
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxNVm43RXV5MWlfOTE5TjdqQjhtd3pzUnRIdmJycExNbXV6REpoRjQ5MlNiRENNemM5SG5VbUhJbnVXenhQXzFhRGgtNXE3QjRWWHhCcTJsZ0lfUW5ZTWNWcjdZQnZSSDM0VVdvVDY0ejBPMklPTUkzdTdXX090b1RQY21nbmdUQUtuZG42RHBxRWdCb05xNkdBT2xUVk1SNWN0cG1NbnhKNlBxSl96T3BzOU91cw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiW0FVX3lxTE1RdV9pa3ZIMmpRWnFlcXRaeTRnSy1zZUp0enVScm1nc0hMX3UwTEdEOG9oQy00UUJiSUR4WENleElGQVVmLXh3ZE10b09nQWphT0IzNHNJb0h3Q0E?oc=5</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr"/>
@@ -1146,12 +1146,12 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Corporate Tax</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
@@ -1161,12 +1161,12 @@
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>UAE extends corporate tax relief for small businesses until 2029 - Khaleej Times</t>
+          <t>FTA Directive No. 5 of 2026 - Crowe</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>News — UAE Corporate Tax</t>
+          <t>News — UAE VAT</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -1176,7 +1176,7 @@
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxNMDNwUlhpclFxaFJkdkkzR0s5MVh4WHZOUDdfZzZtNTBFb2RIcklxMF91Tkp2NGRxRlZMM3BubEZGc0g5LXpsQUhHQy01eGcxTllzc1k1S1NqeFMtYXM4YlBmREttNlhsS0hmd2JXN0l2UjFEQ3B5M1pfRTVpOGw0Z1pPMTNHd0tHQ25ZNjNGZmVaZnhzZUJueE9sQ2dNNGVaUDVjTdIBrAFBVV95cUxNbWJjeHFtRU9DbExyNHRRY1NEUXB2WnZRZ1V2TlFhQ010T3RhSmptR2ItaDhxVnEta0NITUJyS3ppaGgyQ2FkclQwRFhCaWNnLUhNb21YaDVGLWZZNThic2hpN0MzNTI4cXI3RjYtLVUzN3VHanJUUHdYaEFRWUlvS2w5UVdja3pwd1Q4c2pXWHVPZ0xZVmFCcE43eWl1bG10N0s4UXdpVUhpU0tH?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiVkFVX3lxTE40S0RnRzF2d1dBSmNHdkNNQXZQQmlOYWNOSk5OWnlVNUN3ZDB5UHBUV29RXzNvaF9pVFNQZ2FwTUdocGhxMXp1T3gxMUFycGNESFA1bXNR?oc=5</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr"/>
@@ -1191,12 +1191,12 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Corporate Tax</t>
+          <t>VAT</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
@@ -1206,12 +1206,12 @@
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>UAE extends corporate tax relief for small businesses until 2029 - thenationalnews.com</t>
+          <t>Digital currency and VAT: New UAE rules for businesses to consider - thenationalnews.com</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>News — UAE Corporate Tax</t>
+          <t>News — UAE VAT</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
@@ -1221,7 +1221,7 @@
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiwwFBVV95cUxQOFMwcEtFYkFkbWxMRnBqX3Y1M2ZOcnJ4Q1FzTHg2b1NDYnU3dzVWMmMycVdhNzJSbTZhaTZ1bjRpN3RYcm9Gb3VIOUxydjN6anFTMU12SHNNcmt1YkhwSk1RVTV6Yk1yS0wtNm9PbVZLNkxmTVRNd3hEOW1xbXdnTlBiX0VJWWhINEw5MHc1eEk4UHhFZHFOZ04zcnZERDZhLXZJQ0VGWS15N080ZXBQYVhDMFU2al9wN1NlNXN2RnFaZEU?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiugFBVV95cUxQamI1MElzOEtNS1ZjVWR3VGpjZjNUZjBXbjQwZkJIZ3AwOFVqckl0WWFQN2JpaEg5XzRTUTBVMDFOeVhMaUZxYW9GUnBFNW55WnhKd2ZKOVZoekRBWUNqQkp3dGFPZ2JQcWY5SjVlRUJuTURfcVN5aUNXVmthdUh4cHlJbFNHN3lyT1VTU2l2Nk92U09JZFh3eXp0c29jTlJNZW1VLTZBR2h5WmdBTjFuNGczZkZwdDY1QWc?oc=5</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr"/>
@@ -1231,17 +1231,17 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>VAT</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
@@ -1251,12 +1251,12 @@
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>September 1 change: UAE announces new excise price rule for electronic smoking products - Gulf Business</t>
+          <t>Air India turbulence injures passengers on Phuket-Delhi flight - Gulf Business</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>News — FTA Announcements</t>
+          <t>News — UAE Corporate Tax</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -1266,7 +1266,7 @@
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiwAFBVV95cUxNMXNESjR5VDVIQ0Qwb0xKUk1xRlhaTmV2RjNfdVpGaDZZYk0wcjdSbC1RRHBUNkRRaGpNOS1mSjR1blVVRHJ6MzdLeUZXM1lMWURyX21CS25DZFN3engwRWZCOFFLUDJydEEwX0pSa1lLSlNqbVlhdk9pNmtvLUh1QzFubU9RVENUNEl3QVdLc2FkRUV6TGFjZmJwLUtiUVd5dlhjVW1SLU43WFI4eGNfZkJCTXBNaEQySVR3QjZuazA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxOUk92b3hCQVZybGNndXNJOF9ZX0Z3TGl5NnRuXzE5NlBRb3czZXM2SkxXb3ZQSGNOdGo2a2U2b040ZVFDcFBqbzdvaFFZaVdBbFgwQkJOOEhDNzF6VXY1OU9Ca2t2Z1ZnQlhscXNXTVhDaWY3b2lvMUlEWFhkXzVxaDR3b191OUx2aTVKcEttYkFGTjRzRVpnbFJvLUZhYmNLTFJJNg?oc=5</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr"/>
@@ -1276,12 +1276,12 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
@@ -1296,12 +1296,12 @@
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>UAE small businesses claiming tax relief must still file corporate tax returns - Emirates 24|7</t>
+          <t>UAE Business: UAE extends small business relief for corporate tax until December 2029 - Gulf Daily News</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>News — FTA Announcements</t>
+          <t>News — UAE Corporate Tax</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
@@ -1311,7 +1311,7 @@
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxOLXJ6YVV3T2dXazExeU04V09UYlk3NmtYT2d3Z2t1X2RPckN0RjVQZE9oNTljdi1rUUlzTDlMalotZ1JWRS03TWVFWlVVS1hyMVlDUEsxYWQ3RWgtdTdUNzVaZjE5WlhVVUhJcjkyaDFVa28yeEN2ejAtVG43dnduV2NDa0k4czRLby1sU2w2ZHZTcGtPZmpiTjRYWXB2VUExMnhreUktUDBZSkZ4LUxZYW9TYXRJc2s0U1QyMtIB1wFBVV95cUxPNWVmQzRQOEJkZnBCZVFDblE2dkFlX1hGNWlnalJBVk5QREJoU0ZvMXZIM1JJYXdLb2lQZFNnejliekY3Y29nN0tLdTUxQ0h0SUFaSVlpOWhuX3dVaHdjX3NPM1pkd2xlVDRMT1VmTHJ4QV9PbmpWRmVHRFpHZ1lyUF9ZWEJTcFJ2LS1QX0hEa0Y3dnJ4S054S211cWRMWWlHVVd2V19wQnhGa2JVR1ZxSFVNVWJMejdESlFZSkxUMGYwQUlyQkpueDlwb2dJYnlqQnZGNklscw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxNVm43RXV5MWlfOTE5TjdqQjhtd3pzUnRIdmJycExNbXV6REpoRjQ5MlNiRENNemM5SG5VbUhJbnVXenhQXzFhRGgtNXE3QjRWWHhCcTJsZ0lfUW5ZTWNWcjdZQnZSSDM0VVdvVDY0ejBPMklPTUkzdTdXX090b1RQY21nbmdUQUtuZG42RHBxRWdCb05xNkdBT2xUVk1SNWN0cG1NbnhKNlBxSl96T3BzOU91cw?oc=5</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr"/>
@@ -1321,12 +1321,12 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -1341,12 +1341,12 @@
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>UAE releases registration requirements for domestic minimum top-up tax - kpmg.com</t>
+          <t>UAE extends corporate tax relief for small businesses until 2029 - Khaleej Times</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>News — FTA Announcements</t>
+          <t>News — UAE Corporate Tax</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -1356,7 +1356,7 @@
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxPaGJWUy1MU0VZdmd3LTVPTmw0bDYtWlF5a3JCVkFwVnhJRUkxVkdEWUE4X1VZLXg0Tkg4YTlLWHhoOUJYVzJqR3lzUE5Pa1RpSWtjdkRDQ09UeDBoQ3Y2bGlLbkhzTXZ2WlNJeGFSLXNqRUZyRnBfNV9Mbk5UY25hdVZ6VWM2cWRYOEt4bUlnWV9QYkQtOWZudGJaV0ZJZDRVY2JGbTY1T1JTYVhyTGhEdlVuQzlzZkN6ZC1VRQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMipAFBVV95cUxNMDNwUlhpclFxaFJkdkkzR0s5MVh4WHZOUDdfZzZtNTBFb2RIcklxMF91Tkp2NGRxRlZMM3BubEZGc0g5LXpsQUhHQy01eGcxTllzc1k1S1NqeFMtYXM4YlBmREttNlhsS0hmd2JXN0l2UjFEQ3B5M1pfRTVpOGw0Z1pPMTNHd0tHQ25ZNjNGZmVaZnhzZUJueE9sQ2dNNGVaUDVjTdIBrAFBVV95cUxNbWJjeHFtRU9DbExyNHRRY1NEUXB2WnZRZ1V2TlFhQ010T3RhSmptR2ItaDhxVnEta0NITUJyS3ppaGgyQ2FkclQwRFhCaWNnLUhNb21YaDVGLWZZNThic2hpN0MzNTI4cXI3RjYtLVUzN3VHanJUUHdYaEFRWUlvS2w5UVdja3pwd1Q4c2pXWHVPZ0xZVmFCcE43eWl1bG10N0s4UXdpVUhpU0tH?oc=5</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr"/>
@@ -1366,17 +1366,17 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Corporate Tax</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
@@ -1386,12 +1386,12 @@
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>UAE Digital Economy: Why Trust, Not Speed, Now Wins The Race - Menafn</t>
+          <t>UAE extends corporate tax relief for small businesses until 2029 - thenationalnews.com</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>News — UAE E-Invoicing</t>
+          <t>News — UAE Corporate Tax</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -1401,7 +1401,7 @@
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMikAFBVV95cUxNbi1OcWZwSTNNYjBRZkJWS1FodlVGTG5oZHB1T3Q2cGRqazRiZGQzeUtlOVB3VXlhNUM1TnhSdW1MVS1uSng1dGFmTlAzb3ZMNXlod0c5bWo2RkdOTW1idm9JQ3dQNTM5Z3FvZl96WlNuVVh4Mmx5NGFNWXBHVFZoWnUyQU9WT01idllWclJqTXE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiwwFBVV95cUxQOFMwcEtFYkFkbWxMRnBqX3Y1M2ZOcnJ4Q1FzTHg2b1NDYnU3dzVWMmMycVdhNzJSbTZhaTZ1bjRpN3RYcm9Gb3VIOUxydjN6anFTMU12SHNNcmt1YkhwSk1RVTV6Yk1yS0wtNm9PbVZLNkxmTVRNd3hEOW1xbXdnTlBiX0VJWWhINEw5MHc1eEk4UHhFZHFOZ04zcnZERDZhLXZJQ0VGWS15N080ZXBQYVhDMFU2al9wN1NlNXN2RnFaZEU?oc=5</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr"/>
@@ -1416,7 +1416,7 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -1431,12 +1431,12 @@
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>Ministry of Finance sets e-cigarette liquid excise price - Sharjah24</t>
+          <t>September 1 change: UAE announces new excise price rule for electronic smoking products - Gulf Business</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>News — UAE E-Invoicing</t>
+          <t>News — FTA Announcements</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -1446,7 +1446,7 @@
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiWkFVX3lxTFBGY1BCNkVheXBxM3RBdWlPNXVULWVaaWdWM3RWWU9JSWI2T3JVMGlMdl94Ync5ekFqdGU1SzAxeEMwaUhJR1hTejhVTFo4blI2Y1d5QzZUaVgwUQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiwAFBVV95cUxNMXNESjR5VDVIQ0Qwb0xKUk1xRlhaTmV2RjNfdVpGaDZZYk0wcjdSbC1RRHBUNkRRaGpNOS1mSjR1blVVRHJ6MzdLeUZXM1lMWURyX21CS25DZFN3engwRWZCOFFLUDJydEEwX0pSa1lLSlNqbVlhdk9pNmtvLUh1QzFubU9RVENUNEl3QVdLc2FkRUV6TGFjZmJwLUtiUVd5dlhjVW1SLU43WFI4eGNfZkJCTXBNaEQySVR3QjZuazA?oc=5</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr"/>
@@ -1461,12 +1461,12 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Corporate Tax</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
@@ -1476,12 +1476,12 @@
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>CBUAE injects more liquidity into the banking system - EnterpriseAM</t>
+          <t>UAE small businesses claiming tax relief must still file corporate tax returns - Emirates 24|7</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>News — UAE E-Invoicing</t>
+          <t>News — FTA Announcements</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
@@ -1491,7 +1491,7 @@
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxPRVF2amFoSUlsRENGenUxcUlxRU9NeU9QWlJhUkExb1k0cExublF1YUdrM2dJc0FySm9zQmgyQUtKU092bkpYT1I1bUhaMkxGR2o2SFVnckhIR2d4RGQzOUJnb19tZERINThyZ0NrQ1A0WUttandLcmN0QUlUaTFVZ1djMnUxdEp4SmNGMjM1Zl9HX1k?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxOLXJ6YVV3T2dXazExeU04V09UYlk3NmtYT2d3Z2t1X2RPckN0RjVQZE9oNTljdi1rUUlzTDlMalotZ1JWRS03TWVFWlVVS1hyMVlDUEsxYWQ3RWgtdTdUNzVaZjE5WlhVVUhJcjkyaDFVa28yeEN2ejAtVG43dnduV2NDa0k4czRLby1sU2w2ZHZTcGtPZmpiTjRYWXB2VUExMnhreUktUDBZSkZ4LUxZYW9TYXRJc2s0U1QyMtIB1wFBVV95cUxPNWVmQzRQOEJkZnBCZVFDblE2dkFlX1hGNWlnalJBVk5QREJoU0ZvMXZIM1JJYXdLb2lQZFNnejliekY3Y29nN0tLdTUxQ0h0SUFaSVlpOWhuX3dVaHdjX3NPM1pkd2xlVDRMT1VmTHJ4QV9PbmpWRmVHRFpHZ1lyUF9ZWEJTcFJ2LS1QX0hEa0Y3dnJ4S054S211cWRMWWlHVVd2V19wQnhGa2JVR1ZxSFVNVWJMejdESlFZSkxUMGYwQUlyQkpueDlwb2dJYnlqQnZGNklscw?oc=5</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr"/>
@@ -1511,7 +1511,7 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Corporate Tax</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -1521,12 +1521,12 @@
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>The Taxation Society partners with Tally Solutions to strengthen UAE's finance and tax professional community - khaleejtimes.com</t>
+          <t>UAE releases registration requirements for domestic minimum top-up tax - kpmg.com</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>News — UAE E-Invoicing</t>
+          <t>News — FTA Announcements</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -1536,7 +1536,7 @@
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi4gFBVV95cUxNMXRpRGhpQXJvUkZhQU1IcTF6Z0JtLW16cTQ1d24zZWlwQTlPMHNCeG8tY0NLc1JGcXdjT2g5V01YM3hOVmtZYzBJeThiR3hhSDRpdGdwaDhsVC1WMDFTSWN0SWdhc3hiWTRSQmV0blZEZkowYWdoSU1BaUJ6Y01ZZ2ZrWlNRc2JtUllnc0huTF92aWdmbEp4bTRvRV9fN2xTU2dmMjdLSk43ZlFlcEtuWTBKQXdFTU5pMlRnWE55VFBwcTc0STRtcFluS3Ffek1oM2NRQ1dYemVkTktESkJRSVJ30gHqAUFVX3lxTE85ZnVhMjFKMWdhenV1YlFiRGtpVTBIdjRvLVNLRFBjTHBPUnVfeG5sUGxIcWVlSlhUTEVibFV2UXdWbEg5TGNmS3hBYnczSEctV3BBT2pZT3dpcDJUeGczWE9xQ1dweV9hc1hwQnhHQkFWUDRrb0FzV0tVdmZhZ0pLZC14YlVJZjBYQmcwbUZWeG55dnhpOFliT0wxYkQ0bzl1VEhiVUpQNjQ4TVN0bFhPRERROXB5NUZZQ0VRS08tY0VmSDdLRFQzMHZ0dEZtamJ5dmp1OGZ6SmNxQjZrck8wRWs2U1A0TFJZdw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxPaGJWUy1MU0VZdmd3LTVPTmw0bDYtWlF5a3JCVkFwVnhJRUkxVkdEWUE4X1VZLXg0Tkg4YTlLWHhoOUJYVzJqR3lzUE5Pa1RpSWtjdkRDQ09UeDBoQ3Y2bGlLbkhzTXZ2WlNJeGFSLXNqRUZyRnBfNV9Mbk5UY25hdVZ6VWM2cWRYOEt4bUlnWV9QYkQtOWZudGJaV0ZJZDRVY2JGbTY1T1JTYVhyTGhEdlVuQzlzZkN6ZC1VRQ?oc=5</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr"/>
@@ -1551,12 +1551,12 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Corporate Tax</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
@@ -1566,7 +1566,7 @@
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>MoF extends Small Business Relief for corporate tax until end-2029 - Sharjah24</t>
+          <t>UAE Digital Economy: Why Trust, Not Speed, Now Wins The Race - Menafn</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
@@ -1581,7 +1581,7 @@
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiW0FVX3lxTFA4N01YTUZ2UGRGVWdDQ3JDM3JLYWJDanVuckdCLVhuQUdqUFo3clA1cGRoTUtubWNpQ0dTOUFSQk5jYzdGcVFYNkNpQjF4ckFVZ2pBc0FXM1Ffa0k?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMikAFBVV95cUxNbi1OcWZwSTNNYjBRZkJWS1FodlVGTG5oZHB1T3Q2cGRqazRiZGQzeUtlOVB3VXlhNUM1TnhSdW1MVS1uSng1dGFmTlAzb3ZMNXlod0c5bWo2RkdOTW1idm9JQ3dQNTM5Z3FvZl96WlNuVVh4Mmx5NGFNWXBHVFZoWnUyQU9WT01idllWclJqTXE?oc=5</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr"/>
@@ -1601,7 +1601,7 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>VAT</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -1611,7 +1611,7 @@
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>Northern Emirates’ property markets cool off + Sidara locks in USD 1.35 bn in firepower - EnterpriseAM</t>
+          <t>Ministry of Finance sets e-cigarette liquid excise price - Sharjah24</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
@@ -1626,7 +1626,7 @@
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxOMDUxZXd1MElSNXdaNDByLW9jbHFIenJCY21PRnhPMUx4YkdyZ1FMREVxenNWZWZUY2p3MHQ5V2xUQmswZ1RuV1g3Q3RHUzdvOFhvOGpST2diQWIwOXFBeXdzc1lYRl9FRDIxdjBjUVR3Y2VEcUdIWXB0amg4YW5qbklORzFMS3J4VUZGelkybDVZcXc0VHlNck4zTXdjR1N1UzZmSk9vSFFoMDJMVENKMFVlWEdvUTEwZFhiZmdn?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiWkFVX3lxTFBGY1BCNkVheXBxM3RBdWlPNXVULWVaaWdWM3RWWU9JSWI2T3JVMGlMdl94Ync5ekFqdGU1SzAxeEMwaUhJR1hTejhVTFo4blI2Y1d5QzZUaVgwUQ?oc=5</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr"/>
@@ -1646,7 +1646,7 @@
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>E-Invoicing</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
@@ -1656,7 +1656,7 @@
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>ClearTax urges UAE businesses to prioritise execution assurance as e-invoicing decisions gather pace - Gulf News</t>
+          <t>CBUAE injects more liquidity into the banking system - EnterpriseAM</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
@@ -1671,7 +1671,7 @@
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi6wFBVV95cUxPTG13TFpCRmpaaWU3ZGxsVEtqakxUUXhSc0ltWUZfOEUyWTcxWGhOZ2doazNZY1V2LWFnSlp0NHpHTXN4emN6TzFWbGlXT09xU0Q3X25BTmpBVVl0Nl9XMFdRUE9HMy1BU3BMRDFIZ1RITkw4d3BSanluZGFHal9CM3h5dDNtTlBtUG9LYXZZWkhILVZhdUpKTHhUd2lMWmVOdVJrREx4UUF4WjNvTW5hSmtBVjVyQVBpblVKa1hKbjhxRTNUVmpUMVpXOFFJSWx1NUZWUWFMYlY2ZjA2Nml6OGV6X2ZGcVhkQkQ00gH-AUFVX3lxTE12b1Q4Qjd0Rks3U1hqOC1GVTZ5RXRUOXB6eVdVd3RMTEV5Q1pRYVRrc19GaG1qY3FXRGhqMkN3N3c2emJyeTFWbEU2QkRSMHR5aWFzNlctUi1mdi1vamRHMHZoWFZlQlRCbEhrT3BLSXlsTXRfYjY4QjVHblFRU0JnZVhlam4xNEF6d0hQVUtmTHFoYnktSW5LS3dqU2VleEh4azlObnoyUTNPd2E0RWc4U0ZhMkRoc1J1c2R6VGJhc1lSYTF0cjhzdnY0Q0tvYk81YnY5UE5CdnBXZTVNQXE4UlZwMkFjbUREaEtRNlF2MWJYVFhaOTFJNTZRUlJn?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxPRVF2amFoSUlsRENGenUxcUlxRU9NeU9QWlJhUkExb1k0cExublF1YUdrM2dJc0FySm9zQmgyQUtKU092bkpYT1I1bUhaMkxGR2o2SFVnckhIR2d4RGQzOUJnb19tZERINThyZ0NrQ1A0WUttandLcmN0QUlUaTFVZ1djMnUxdEp4SmNGMjM1Zl9HX1k?oc=5</t>
         </is>
       </c>
       <c r="I27" s="2" t="inlineStr"/>
@@ -1686,7 +1686,7 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
@@ -1701,7 +1701,7 @@
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>UAE extends small business tax relief until 2029 - theaccountant-online.com</t>
+          <t>The Taxation Society partners with Tally Solutions to strengthen UAE's finance and tax professional community - khaleejtimes.com</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
@@ -1716,7 +1716,7 @@
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxOMTA1XzlxbnpmYjNMcU01VXV1RjdMOHFuMi1CSVNMYXlaNW9kb2ZMSXZXOEZ1dDlqbmRLR2hXQjNrMDdlaU4teDVRTG1CMmJsY0lDU3V0SWxRZE4tWXZXbV9pR2o5THFMREVyZ3VpY1pTYVhFeUJza1MwOWtVYXB1ckwxQlBRdVF6eURUUHlkblhUNnNoQ3c?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi4gFBVV95cUxNMXRpRGhpQXJvUkZhQU1IcTF6Z0JtLW16cTQ1d24zZWlwQTlPMHNCeG8tY0NLc1JGcXdjT2g5V01YM3hOVmtZYzBJeThiR3hhSDRpdGdwaDhsVC1WMDFTSWN0SWdhc3hiWTRSQmV0blZEZkowYWdoSU1BaUJ6Y01ZZ2ZrWlNRc2JtUllnc0huTF92aWdmbEp4bTRvRV9fN2xTU2dmMjdLSk43ZlFlcEtuWTBKQXdFTU5pMlRnWE55VFBwcTc0STRtcFluS3Ffek1oM2NRQ1dYemVkTktESkJRSVJ30gHqAUFVX3lxTE85ZnVhMjFKMWdhenV1YlFiRGtpVTBIdjRvLVNLRFBjTHBPUnVfeG5sUGxIcWVlSlhUTEVibFV2UXdWbEg5TGNmS3hBYnczSEctV3BBT2pZT3dpcDJUeGczWE9xQ1dweV9hc1hwQnhHQkFWUDRrb0FzV0tVdmZhZ0pLZC14YlVJZjBYQmcwbUZWeG55dnhpOFliT0wxYkQ0bzl1VEhiVUpQNjQ4TVN0bFhPRERROXB5NUZZQ0VRS08tY0VmSDdLRFQzMHZ0dEZtamJ5dmp1OGZ6SmNxQjZrck8wRWs2U1A0TFJZdw?oc=5</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr"/>
@@ -1731,12 +1731,12 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>VAT</t>
+          <t>Corporate Tax</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
@@ -1746,7 +1746,7 @@
       </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
-          <t>Sovos Announces 2026 Partner of the Year Award Winners, Recognizing Excellence in Strategic Collaboration and Innovation - Business Wire</t>
+          <t>MoF extends Small Business Relief for corporate tax until end-2029 - Sharjah24</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
@@ -1761,7 +1761,7 @@
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMihwJBVV95cUxQRzJIdmQ3VjZqenlUTldPal9HNXdxdTJibTJHWFBhMVBMTWcxbm0yeUhJYzVLd0Z3Yl9pdE1LQzREWm13dXE4ZG1abDFuRkZIdHhIcm4zYXVoOXZIS01KNW5xRU04SUVwMlRnZlBxb3BYQkJMQ01CeXhabEI5U1VfSlpad0ROaVNnTUVnUll2WFhwMkxUa2tidGRxTDlMRm93SlAxVkNoWW84Zk1oeFFoNVdnOWRBZERIZzNSdnVDMGpHZ0MzSXlxZ1JXc2hodEY0aXNoRkNBRldSOGdxSkowdmFoTEplTjBtOUVfeWFtNmpzeDZtR3J2bVk4UWthWFR5VjJRbEM2NA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiW0FVX3lxTFA4N01YTUZ2UGRGVWdDQ3JDM3JLYWJDanVuckdCLVhuQUdqUFo3clA1cGRoTUtubWNpQ0dTOUFSQk5jYzdGcVFYNkNpQjF4ckFVZ2pBc0FXM1Ffa0k?oc=5</t>
         </is>
       </c>
       <c r="I29" s="2" t="inlineStr"/>
@@ -1791,7 +1791,7 @@
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>UAE E Invoicing Guidelines Updated to Version 1.1 - Crowe</t>
+          <t>Northern Emirates’ property markets cool off + Sidara locks in USD 1.35 bn in firepower - EnterpriseAM</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
@@ -1806,7 +1806,7 @@
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMigAFBVV95cUxQOGUxa2xtLVY1ejE0azVCMEZSa3lxNHZmajhUdzh5LTQ5NGRqVk5oenBzNmJUSk44X1B0elZ5aDI5YVl4VHpLb2RzdEFRYW9IVmR5dHpOaE1JbWVoNzdvQVpsR0xIalA1MHBaR1NNOVpVSHUyX2t4R0dIVmZiWHlXWg?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxOMDUxZXd1MElSNXdaNDByLW9jbHFIenJCY21PRnhPMUx4YkdyZ1FMREVxenNWZWZUY2p3MHQ5V2xUQmswZ1RuV1g3Q3RHUzdvOFhvOGpST2diQWIwOXFBeXdzc1lYRl9FRDIxdjBjUVR3Y2VEcUdIWXB0amg4YW5qbklORzFMS3J4VUZGelkybDVZcXc0VHlNck4zTXdjR1N1UzZmSk9vSFFoMDJMVENKMFVlWEdvUTEwZFhiZmdn?oc=5</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr"/>
@@ -1826,7 +1826,7 @@
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>VAT, E-Invoicing</t>
+          <t>E-Invoicing</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
@@ -1836,7 +1836,7 @@
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>Congo Republic e-invoicing launched - vatcalc.com</t>
+          <t>ClearTax urges UAE businesses to prioritise execution assurance as e-invoicing decisions gather pace - Gulf News</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
@@ -1851,7 +1851,7 @@
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMijgFBVV95cUxOLTlBQUhqTDJya1ZpUmx5Y0lPRlRHb0VpWW5GYWVBc1JkTGRFbFl0b3N5UGJSdEdXRmwxdld1RlhqSWVremtIU1pWSHNXb2ROejA2TzJYcF9RX29TQVN1akJ5d0cxWFplcmJPYUJTRDgzU2FzenRzMzJldUsyaE9rbzlVUmJMSEc5M1pzSGtR?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi6wFBVV95cUxPTG13TFpCRmpaaWU3ZGxsVEtqakxUUXhSc0ltWUZfOEUyWTcxWGhOZ2doazNZY1V2LWFnSlp0NHpHTXN4emN6TzFWbGlXT09xU0Q3X25BTmpBVVl0Nl9XMFdRUE9HMy1BU3BMRDFIZ1RITkw4d3BSanluZGFHal9CM3h5dDNtTlBtUG9LYXZZWkhILVZhdUpKTHhUd2lMWmVOdVJrREx4UUF4WjNvTW5hSmtBVjVyQVBpblVKa1hKbjhxRTNUVmpUMVpXOFFJSWx1NUZWUWFMYlY2ZjA2Nml6OGV6X2ZGcVhkQkQ00gH-AUFVX3lxTE12b1Q4Qjd0Rks3U1hqOC1GVTZ5RXRUOXB6eVdVd3RMTEV5Q1pRYVRrc19GaG1qY3FXRGhqMkN3N3c2emJyeTFWbEU2QkRSMHR5aWFzNlctUi1mdi1vamRHMHZoWFZlQlRCbEhrT3BLSXlsTXRfYjY4QjVHblFRU0JnZVhlam4xNEF6d0hQVUtmTHFoYnktSW5LS3dqU2VleEh4azlObnoyUTNPd2E0RWc4U0ZhMkRoc1J1c2R6VGJhc1lSYTF0cjhzdnY0Q0tvYk81YnY5UE5CdnBXZTVNQXE4UlZwMkFjbUREaEtRNlF2MWJYVFhaOTFJNTZRUlJn?oc=5</t>
         </is>
       </c>
       <c r="I31" s="2" t="inlineStr"/>
@@ -1866,7 +1866,7 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
@@ -1881,12 +1881,12 @@
       </c>
       <c r="E32" s="3" t="inlineStr">
         <is>
-          <t>Corporate Governance in the UAE - Crowe</t>
+          <t>UAE extends small business tax relief until 2029 - theaccountant-online.com</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>News — UAE Transfer Pricing</t>
+          <t>News — UAE E-Invoicing</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
@@ -1896,7 +1896,7 @@
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMibkFVX3lxTE4weWRYb0VETFpvMjdhUG9BbU5Wb2JXbzNkLVpxSC1VZHhwYjMwT0F2OFNvQkJNQTFkOG1OamVFZWU0NWpVN3hHb0lldkJWLV9GeThwSjdzNlpnQXp0VDdQbkpnSWFFU3lacVJOeXl3?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMilgFBVV95cUxOMTA1XzlxbnpmYjNMcU01VXV1RjdMOHFuMi1CSVNMYXlaNW9kb2ZMSXZXOEZ1dDlqbmRLR2hXQjNrMDdlaU4teDVRTG1CMmJsY0lDU3V0SWxRZE4tWXZXbV9pR2o5THFMREVyZ3VpY1pTYVhFeUJza1MwOWtVYXB1ckwxQlBRdVF6eURUUHlkblhUNnNoQ3c?oc=5</t>
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr"/>
@@ -1916,7 +1916,7 @@
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>VAT</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
@@ -1926,12 +1926,12 @@
       </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
-          <t>Shopping online in the UAE? Tourists can now claim tax refunds on Noon orders - The Global Filipino Magazine</t>
+          <t>Sovos Announces 2026 Partner of the Year Award Winners, Recognizing Excellence in Strategic Collaboration and Innovation - Business Wire</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>News — UAE VAT</t>
+          <t>News — UAE E-Invoicing</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
@@ -1941,7 +1941,7 @@
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxNa1BKRVpJRVZCZm5VNVp2d3h4Rl92ejg0aml0Qy1pTUotYTZ4ZHlaeURMcnRacE9Zc0J2TWt4VktTQWdFV3BlNXBzWmlfMXFEZFRiYWRIMmV3X3ItaWc0T3pzOG52THI4c1RQaDY1RWdNbXItTTUtdlFTS1d6SUpZTVlXM2lOTWtLWXF6TGNSRE9OWkJQSUs3UXFoSEtOa2NpNEJLeTFOektldFVUVHk4cFJCSE5Qdw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMihwJBVV95cUxQRzJIdmQ3VjZqenlUTldPal9HNXdxdTJibTJHWFBhMVBMTWcxbm0yeUhJYzVLd0Z3Yl9pdE1LQzREWm13dXE4ZG1abDFuRkZIdHhIcm4zYXVoOXZIS01KNW5xRU04SUVwMlRnZlBxb3BYQkJMQ01CeXhabEI5U1VfSlpad0ROaVNnTUVnUll2WFhwMkxUa2tidGRxTDlMRm93SlAxVkNoWW84Zk1oeFFoNVdnOWRBZERIZzNSdnVDMGpHZ0MzSXlxZ1JXc2hodEY0aXNoRkNBRldSOGdxSkowdmFoTEplTjBtOUVfeWFtNmpzeDZtR3J2bVk4UWthWFR5VjJRbEM2NA?oc=5</t>
         </is>
       </c>
       <c r="I33" s="2" t="inlineStr"/>
@@ -1956,12 +1956,12 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>VAT</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
@@ -1971,12 +1971,12 @@
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
-          <t>Number of retail outlets connected to Digital Tourist VAT Refund System reaches more than 19,300 - Big News Network.com</t>
+          <t>UAE E Invoicing Guidelines Updated to Version 1.1 - Crowe</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>News — UAE VAT</t>
+          <t>News — UAE E-Invoicing</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -1986,7 +1986,7 @@
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi2AFBVV95cUxNUjRVVzdLOXJQTXpUZDhqeWlQNDAwVDV2ZmJqd3h4cW5ZbXc0cHEzZGJBSWlLOTk0ZlFFbXlVSThCUEtxcGFqUHYzSlRmeXF0bC1XQ1J3VVhKUUkzeVBfNTc4cmQwNmlRYldwUU01YXpmc0pxT0daNWRpRUwtM0N3MlBBR09rRldZZlA5bXVJOXVTcVZSeE5ldWRHSWhna0ZfTTNwZWEwODlFTXRRYnRhOVJVcHJ3dDRuSnZtQlBhc0NMa2dhSzk4b1lBWEx5Uk5Ld2RMaFdmNUY?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMigAFBVV95cUxQOGUxa2xtLVY1ejE0azVCMEZSa3lxNHZmajhUdzh5LTQ5NGRqVk5oenBzNmJUSk44X1B0elZ5aDI5YVl4VHpLb2RzdEFRYW9IVmR5dHpOaE1JbWVoNzdvQVpsR0xIalA1MHBaR1NNOVpVSHUyX2t4R0dIVmZiWHlXWg?oc=5</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr"/>
@@ -2001,12 +2001,12 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>VAT</t>
+          <t>VAT, E-Invoicing</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
@@ -2016,12 +2016,12 @@
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>UAE tourists can claim VAT refunds at 19,340 stores and on Noon purchases - Gulf News</t>
+          <t>Congo Republic e-invoicing launched - vatcalc.com</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>News — UAE VAT</t>
+          <t>News — UAE E-Invoicing</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
@@ -2031,7 +2031,7 @@
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxQeDRPcDE4QjJaSFU3Qm1wRGVaWXl6cjY2c3YyVDF3TmtqN1RYMkh0WDdoSm56QmlXU21xSllRQWt4WHNFU09vUWZpTEd3dVVMb0UxNy0yZG1ucUF6aXhIZ2dWVXpkVjVqa2hHUGN3VHNZWEticFZMXzNfb2NzaVpwOFFkOVAtNDhBY0xjSUo3bkh0WUg2ZEJ4Q0JDU05Td0FTLWlUWXNfN2JKeGJsTEg3NGFDMzNwT21JZTFGT0V30gHQAUFVX3lxTE9wdElvSG52YzNWWUt6WGJaRkp0LXpmVHpQTFV4WHczVkQtOUhOMWpqRzd2UjgyQjNOSWdMT3QwM1luZzdtNWhXdU91R2lqS0FKcG1hUGExZ1QxWG1SSUo2cWZSWll0bjdpQ2pBOXFjTUMxcjJma0RraGlVbjNjajZRM0h4OVZfM0FUQXNERTQzQm1TS29QVjdiQzM2T19naktoTXhfQ1pvNmx4U2IxVkkxUWF5QmZ4QUxmMXB2bFVvR2RVWm10bjE2SlNaRzJ2VEU?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMijgFBVV95cUxOLTlBQUhqTDJya1ZpUmx5Y0lPRlRHb0VpWW5GYWVBc1JkTGRFbFl0b3N5UGJSdEdXRmwxdld1RlhqSWVremtIU1pWSHNXb2ROejA2TzJYcF9RX29TQVN1akJ5d0cxWFplcmJPYUJTRDgzU2FzenRzMzJldUsyaE9rbzlVUmJMSEc5M1pzSGtR?oc=5</t>
         </is>
       </c>
       <c r="I35" s="2" t="inlineStr"/>
@@ -2046,12 +2046,12 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>VAT</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
@@ -2061,12 +2061,12 @@
       </c>
       <c r="E36" s="3" t="inlineStr">
         <is>
-          <t>Retail outlets linked to UAE's Digital Tourist VAT Refund System exceed 19,300 - Emirates 24|7</t>
+          <t>Corporate Governance in the UAE - Crowe</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>News — UAE VAT</t>
+          <t>News — UAE Transfer Pricing</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
@@ -2076,7 +2076,7 @@
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiugFBVV95cUxOcXRBMGsxX1Q5SkJXcEFwWnV3c0VVc19jUnRkWU5yMVlPelltaEhvOWNLcEJxYi1KUExWMVlmZE1FOExZYklsRHU4N3lQZGppMDRnYUFaRU1OWHdwaVpiWWowOENidVJjbDFPeTQyQklzOGM5bXhQbDJrRFg2TkR6bUplTzJNZzl2M3dJT2FEeHVTTVNtTml6UEdoZUFDcVRCZWFHMGg1ejZoSWI1UWFCLV9zREotcmF3V0HSAdQBQVVfeXFMT3Q0RFN0V3FRSlNWV20tMm5hY1N5VHBVWmxzdnZGVXIwZU92VTZVRDVUVkRZM0Q1U1ZNZzFRcFlEWTc2ckk0UjZhcEN4YmZIZndTd284ZDQ3Z2Z4OS1mVGFUX2RwRzgyMWViTjEyQ19wdUxucXEtZWtFRm5tOWpId1VYYlRmd1Rkc2tlb3Q3THR0THZxZWt3Q1ZyTGVvZ2hUUzZPeTBPSzlER3FXR0ZvUnJiWk5vdlpwYlYxdmZjZnNTVEQxM3hSY1pyTGV5Qkk2d2lrejQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMibkFVX3lxTE4weWRYb0VETFpvMjdhUG9BbU5Wb2JXbzNkLVpxSC1VZHhwYjMwT0F2OFNvQkJNQTFkOG1OamVFZWU0NWpVN3hHb0lldkJWLV9GeThwSjdzNlpnQXp0VDdQbkpnSWFFU3lacVJOeXl3?oc=5</t>
         </is>
       </c>
       <c r="I36" s="2" t="inlineStr"/>
@@ -2091,12 +2091,12 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>VAT</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
@@ -2106,7 +2106,7 @@
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t>Indians, Russians, Turks top list of tourists claiming the most VAT refunds in UAE - khaleejtimes.com</t>
+          <t>Shopping online in the UAE? Tourists can now claim tax refunds on Noon orders - The Global Filipino Magazine</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
@@ -2121,7 +2121,7 @@
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiugFBVV95cUxPek9sY1dJUkpRblhiYnJDdDExOW1yREdXd1oyZ1Yxb0FnZlBYNTd3SUxGWnVMenlZVGlqRlIxLUszNk1Jd3BpcF9rVE9XLVF1OWdhY01fd0gteTJFRkVJLVREMjl4ZVRGZHJacUxJREpRN3UxdHFncGhITEQ0MnUzTkhKY2FSZnBnaFUzZDEyRnZOdG1hOWVFX2FLNG9Ca1lGekQzcllxd0FqTUhvTTRZM3MxcElQV0JaMWfSAcIBQVVfeXFMT2FPTEx4WGUzNUNhZWdBa1MzVU5GN1p3SkRwM0o5TWlqenhqVTNhR1Z0bThyN0laMS1tOUhfaG1qMmZpQi1pT3lTNEhKT2l3SklKZ1E3MXkyYVBrMnUwOTh1Y2RxSkFISUdlT1B6Qm1tTV9CUV9YM0xwcTJ2NzVmWUcxaFJ2YzhYeVBjZG1WSG9vcVc2N2tqRzNreHFwWVpaaUdncndzVEVLaE8zeHczU0Jvdl9FazU2NE1CNWZqQmZmekE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMitgFBVV95cUxNa1BKRVpJRVZCZm5VNVp2d3h4Rl92ejg0aml0Qy1pTUotYTZ4ZHlaeURMcnRacE9Zc0J2TWt4VktTQWdFV3BlNXBzWmlfMXFEZFRiYWRIMmV3X3ItaWc0T3pzOG52THI4c1RQaDY1RWdNbXItTTUtdlFTS1d6SUpZTVlXM2lOTWtLWXF6TGNSRE9OWkJQSUs3UXFoSEtOa2NpNEJLeTFOektldFVUVHk4cFJCSE5Qdw?oc=5</t>
         </is>
       </c>
       <c r="I37" s="2" t="inlineStr"/>
@@ -2136,7 +2136,7 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -2151,7 +2151,7 @@
       </c>
       <c r="E38" s="3" t="inlineStr">
         <is>
-          <t>Tourists can now claim VAT refunds at 19,300 retail outlets across the UAE - Gulf Business</t>
+          <t>Number of retail outlets connected to Digital Tourist VAT Refund System reaches more than 19,300 - Big News Network.com</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
@@ -2166,7 +2166,7 @@
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxQV2tyUkVhVzNVUlZ0QW9LdW5PWV9OTEVSN1FHU2c0Um9qbTRDNXFIdmZUaERGcDFPUkkyTVpzWXBQblJHb1VzVERybTh5WkIzcnRoRFo1ZVBicVRMQXpFZXB3VVJRQVZ6UDNNZDItT1RuTXcxYWxtSU1PaGlPNTFNUnpzLXBGX2QxSy1WVjU4alg4Q0dEWmY4WFZ6cEt1a1FZQXpRODFFN0xRT3VwSWFfNw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMi2AFBVV95cUxNUjRVVzdLOXJQTXpUZDhqeWlQNDAwVDV2ZmJqd3h4cW5ZbXc0cHEzZGJBSWlLOTk0ZlFFbXlVSThCUEtxcGFqUHYzSlRmeXF0bC1XQ1J3VVhKUUkzeVBfNTc4cmQwNmlRYldwUU01YXpmc0pxT0daNWRpRUwtM0N3MlBBR09rRldZZlA5bXVJOXVTcVZSeE5ldWRHSWhna0ZfTTNwZWEwODlFTXRRYnRhOVJVcHJ3dDRuSnZtQlBhc0NMa2dhSzk4b1lBWEx5Uk5Ld2RMaFdmNUY?oc=5</t>
         </is>
       </c>
       <c r="I38" s="2" t="inlineStr"/>
@@ -2196,7 +2196,7 @@
       </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
-          <t>UAE tourists can now claim VAT refunds on eligible Noon online shopping purchases - Arabian Business</t>
+          <t>UAE tourists can claim VAT refunds at 19,340 stores and on Noon purchases - Gulf News</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
@@ -2211,7 +2211,7 @@
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxNSk0xOTlEQk5DQm4tczlCUE1jZ1dmamdsaUQ2TUYwWnlNd2JHMjhhVXZVUF8wNGpSVUFRNXhvU01pY01FMlUwWEt0anFyS3Q3QS0wa3BjZE1YLWtkWkpYeUJxVmlaSUhQM0Z3Mk9odUFYenhNRnBZeUkyQ0doNWJ2VGUySGY2dG9kMnlJaWhuWEMzb25aWjA1VXZkLWRwelk1MXJjbjBrV2F1Z29KZTJ3?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMivgFBVV95cUxQeDRPcDE4QjJaSFU3Qm1wRGVaWXl6cjY2c3YyVDF3TmtqN1RYMkh0WDdoSm56QmlXU21xSllRQWt4WHNFU09vUWZpTEd3dVVMb0UxNy0yZG1ucUF6aXhIZ2dWVXpkVjVqa2hHUGN3VHNZWEticFZMXzNfb2NzaVpwOFFkOVAtNDhBY0xjSUo3bkh0WUg2ZEJ4Q0JDU05Td0FTLWlUWXNfN2JKeGJsTEg3NGFDMzNwT21JZTFGT0V30gHQAUFVX3lxTE9wdElvSG52YzNWWUt6WGJaRkp0LXpmVHpQTFV4WHczVkQtOUhOMWpqRzd2UjgyQjNOSWdMT3QwM1luZzdtNWhXdU91R2lqS0FKcG1hUGExZ1QxWG1SSUo2cWZSWll0bjdpQ2pBOXFjTUMxcjJma0RraGlVbjNjajZRM0h4OVZfM0FUQXNERTQzQm1TS29QVjdiQzM2T19naktoTXhfQ1pvNmx4U2IxVkkxUWF5QmZ4QUxmMXB2bFVvR2RVWm10bjE2SlNaRzJ2VEU?oc=5</t>
         </is>
       </c>
       <c r="I39" s="2" t="inlineStr"/>
@@ -2241,7 +2241,7 @@
       </c>
       <c r="E40" s="3" t="inlineStr">
         <is>
-          <t>FTA issues five binding VAT directives on tax transactions - kpmg.com</t>
+          <t>Retail outlets linked to UAE's Digital Tourist VAT Refund System exceed 19,300 - Emirates 24|7</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
@@ -2256,7 +2256,7 @@
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxQQXptRUZOQlpWYUZiNzd1QThPVDhlUGM3TF9PU3NKZjUyS2lucEZLUUFKZFpfZVhXLWxteTBKbU1OVEU1WXdPVlViT2ZBb2h5dmlHa0Z2bjd0SzMxa1p6TzF0ajhuVFVSaUpkczUxd1lzeGVCeDNwRnpPbXJVNVNGWHB4UTcwR2dCYTJoWTVSYkJGQmxRZE42cXNmOExtclgxR28tUUdYVFRzaE92?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiugFBVV95cUxOcXRBMGsxX1Q5SkJXcEFwWnV3c0VVc19jUnRkWU5yMVlPelltaEhvOWNLcEJxYi1KUExWMVlmZE1FOExZYklsRHU4N3lQZGppMDRnYUFaRU1OWHdwaVpiWWowOENidVJjbDFPeTQyQklzOGM5bXhQbDJrRFg2TkR6bUplTzJNZzl2M3dJT2FEeHVTTVNtTml6UEdoZUFDcVRCZWFHMGg1ejZoSWI1UWFCLV9zREotcmF3V0HSAdQBQVVfeXFMT3Q0RFN0V3FRSlNWV20tMm5hY1N5VHBVWmxzdnZGVXIwZU92VTZVRDVUVkRZM0Q1U1ZNZzFRcFlEWTc2ckk0UjZhcEN4YmZIZndTd284ZDQ3Z2Z4OS1mVGFUX2RwRzgyMWViTjEyQ19wdUxucXEtZWtFRm5tOWpId1VYYlRmd1Rkc2tlb3Q3THR0THZxZWt3Q1ZyTGVvZ2hUUzZPeTBPSzlER3FXR0ZvUnJiWk5vdlpwYlYxdmZjZnNTVEQxM3hSY1pyTGV5Qkk2d2lrejQ?oc=5</t>
         </is>
       </c>
       <c r="I40" s="2" t="inlineStr"/>
@@ -2271,12 +2271,12 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>Corporate Tax</t>
+          <t>VAT</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
@@ -2286,12 +2286,12 @@
       </c>
       <c r="E41" s="3" t="inlineStr">
         <is>
-          <t>UAE extends Corporate Tax Small Business Relief until end of 2029 - travelsdubai.com</t>
+          <t>Indians, Russians, Turks top list of tourists claiming the most VAT refunds in UAE - khaleejtimes.com</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>News — UAE Corporate Tax</t>
+          <t>News — UAE VAT</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
@@ -2301,7 +2301,7 @@
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMingFBVV95cUxOYzFrN28yN3RDREhxYV9CVHl3UGU1NlpvSFJqaHJGWVpraVhEOEtqTnZVQk1OTjVjX1djWENocHdtYy1WY1dBSHZncjg3aGxWOXlwcFktaVVxYzBmZllLbzBaLUUxSEpyNW1HX3V5MG9YMWhTcjNfcnZxQ1JKRHZkMjlYSjlmUHk1SGFEYy0tYmlqWE96ajBqUnNSS19TUQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiugFBVV95cUxPek9sY1dJUkpRblhiYnJDdDExOW1yREdXd1oyZ1Yxb0FnZlBYNTd3SUxGWnVMenlZVGlqRlIxLUszNk1Jd3BpcF9rVE9XLVF1OWdhY01fd0gteTJFRkVJLVREMjl4ZVRGZHJacUxJREpRN3UxdHFncGhITEQ0MnUzTkhKY2FSZnBnaFUzZDEyRnZOdG1hOWVFX2FLNG9Ca1lGekQzcllxd0FqTUhvTTRZM3MxcElQV0JaMWfSAcIBQVVfeXFMT2FPTEx4WGUzNUNhZWdBa1MzVU5GN1p3SkRwM0o5TWlqenhqVTNhR1Z0bThyN0laMS1tOUhfaG1qMmZpQi1pT3lTNEhKT2l3SklKZ1E3MXkyYVBrMnUwOTh1Y2RxSkFISUdlT1B6Qm1tTV9CUV9YM0xwcTJ2NzVmWUcxaFJ2YzhYeVBjZG1WSG9vcVc2N2tqRzNreHFwWVpaaUdncndzVEVLaE8zeHczU0Jvdl9FazU2NE1CNWZqQmZmekE?oc=5</t>
         </is>
       </c>
       <c r="I41" s="2" t="inlineStr"/>
@@ -2316,7 +2316,7 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
@@ -2331,12 +2331,12 @@
       </c>
       <c r="E42" s="3" t="inlineStr">
         <is>
-          <t>UAE seizes 3.58 million non-compliant excise goods - Gulf News</t>
+          <t>Tourists can now claim VAT refunds at 19,300 retail outlets across the UAE - Gulf Business</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>News — UAE Corporate Tax</t>
+          <t>News — UAE VAT</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
@@ -2346,7 +2346,7 @@
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMipwFBVV95cUxOOF9vUDk3UXlsY19FUWtOOEJ2V3Awam9fY09zeS1seXpTUUt2Y05TQlVUVjlwYlVuX2hRN3JBM095eTlqZ3pxWWx5ZWJzUzV1bGdCQ21JMzd1bjRIMGRMdHpiZWVOM1lmOVdtSXlicW4wYUNoYjMySjFTNl9OTnRvYWZycGdhODlTcU9sQUpwUEdJcnltNF9nSXpBWkpJbjF0VG1qeVJqTdIBugFBVV95cUxPMDVISGFVMTVqWFFiS0VMTmlzZzlyWXRVUl9BTjBGaWgtS21lN05BdlppYlVNQkNtYmZWaHRIczNlSWRmbXBBdG9zamlobjFhTFh6R2lYZFJ1RUtKWGZqOWpNd21LTmNxaUF1SjVIUm9UNjF6cmwxUGY2ZHFIVHBFdVJNMXcyeFp3dUZ2V1hpVmtnRmZOY29nLWNWQmxsQ0tHUzd0RjRyRUlZeW1adThtZEpPVl9KT1pFRUE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxQV2tyUkVhVzNVUlZ0QW9LdW5PWV9OTEVSN1FHU2c0Um9qbTRDNXFIdmZUaERGcDFPUkkyTVpzWXBQblJHb1VzVERybTh5WkIzcnRoRFo1ZVBicVRMQXpFZXB3VVJRQVZ6UDNNZDItT1RuTXcxYWxtSU1PaGlPNTFNUnpzLXBGX2QxSy1WVjU4alg4Q0dEWmY4WFZ6cEt1a1FZQXpRODFFN0xRT3VwSWFfNw?oc=5</t>
         </is>
       </c>
       <c r="I42" s="2" t="inlineStr"/>
@@ -2361,12 +2361,12 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>Corporate Tax</t>
+          <t>VAT</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
@@ -2376,12 +2376,12 @@
       </c>
       <c r="E43" s="3" t="inlineStr">
         <is>
-          <t>UAE Extends Small Business Relief for Corporate Tax to 2029 - tbreak.com</t>
+          <t>UAE tourists can now claim VAT refunds on eligible Noon online shopping purchases - Arabian Business</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>News — UAE Corporate Tax</t>
+          <t>News — UAE VAT</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
@@ -2391,7 +2391,7 @@
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMifEFVX3lxTE9icS1QSXhYc09ROHVJdzRtdXJTMEdLa0o5Mm5TZ3VxR002a3lTeFR5anZqRmNtcVEyQWxfQ050UFVOZnFBcFdwT1VoNGlVZU9xYkY2WkM5SlpSSnp6QkpHck5rTUxqOXNjNjM0UmFTQkFfOXZySFFON1pCSXc?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxNSk0xOTlEQk5DQm4tczlCUE1jZ1dmamdsaUQ2TUYwWnlNd2JHMjhhVXZVUF8wNGpSVUFRNXhvU01pY01FMlUwWEt0anFyS3Q3QS0wa3BjZE1YLWtkWkpYeUJxVmlaSUhQM0Z3Mk9odUFYenhNRnBZeUkyQ0doNWJ2VGUySGY2dG9kMnlJaWhuWEMzb25aWjA1VXZkLWRwelk1MXJjbjBrV2F1Z29KZTJ3?oc=5</t>
         </is>
       </c>
       <c r="I43" s="2" t="inlineStr"/>
@@ -2406,12 +2406,12 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Corporate Tax</t>
+          <t>VAT</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
@@ -2421,12 +2421,12 @@
       </c>
       <c r="E44" s="3" t="inlineStr">
         <is>
-          <t>UAE extends corporate tax relief for small businesses until end of 2029 - Gulf News</t>
+          <t>FTA issues five binding VAT directives on tax transactions - kpmg.com</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>News — UAE Corporate Tax</t>
+          <t>News — UAE VAT</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
@@ -2436,7 +2436,7 @@
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMixgFBVV95cUxNNEo4Tm9qN1dERmwzZ0tMR0ZOSUVQTkpOTTNiTDc1U2VaSTkyRkExekRzRjUzb2xrelYzV0oydU1qS2JCbHJXd1hxeWhPdmtUN1UtcXRCOHZpSXBxMlBMdFRKbDNxYlNFaVdwRXROTUVxWC1tZUpObDVIZzNVUDEzSUZpNkIxN3ctTDRNWU9xOUx6QXZieFdVV1hkNHhlcldHUzY5b21BZ1J2VTVhMlN2a1V5V1dJRkw1OTItdWo5Qzk5N2lPX1HSAdgBQVVfeXFMTmRQM08wYWhkelVySDhudHZWLWQyZ2lyUG9TNEJhWVV6ejAybDV6QXdvUFR5ZndxZldxWHVDMjRKVm1Ndm0yeE1HZHo1LXoyVFBzMkhuUDZESEw5RUFIaWlfNEdObjNxRlc4VFpOZVQ3RDhhellsdEpYN3pLVzl1d1Fva3R0RWpDb0d5cVN0Z3I3emowS2tNbkplWTh1Z2NvVkRMd0R3STNWV3hrUVFtd3hxdjQxWjI2ZU4wVE9JTzlsWVUwYXlPTmU4YWJmazMxQk93MHVHbGZE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMirAFBVV95cUxQQXptRUZOQlpWYUZiNzd1QThPVDhlUGM3TF9PU3NKZjUyS2lucEZLUUFKZFpfZVhXLWxteTBKbU1OVEU1WXdPVlViT2ZBb2h5dmlHa0Z2bjd0SzMxa1p6TzF0ajhuVFVSaUpkczUxd1lzeGVCeDNwRnpPbXJVNVNGWHB4UTcwR2dCYTJoWTVSYkJGQmxRZE42cXNmOExtclgxR28tUUdYVFRzaE92?oc=5</t>
         </is>
       </c>
       <c r="I44" s="2" t="inlineStr"/>
@@ -2451,7 +2451,7 @@
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
@@ -2466,7 +2466,7 @@
       </c>
       <c r="E45" s="3" t="inlineStr">
         <is>
-          <t>Small businesses in UAE urged to file corporate tax returns before deadline, says FTA - khaleejtimes.com</t>
+          <t>UAE extends Corporate Tax Small Business Relief until end of 2029 - travelsdubai.com</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
@@ -2481,7 +2481,7 @@
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxOWnJlYmRmRm4xdy0xZ0toMUNUbnhTd3A5UW1pVzhFeXhIM2txamo4NU5qYVYwZGlQcEYwLTJhelBkOEdHajRYSE5PRnZtdmxGWmc0R2JlUVk0eVc0aW53NzdlM08zeWFzTUNocU9UcnY3UTNhTHVzZHhjRXFPZ0ZMMHMyRExEcjFiVVhKVzMxYk9FSHUxdERQRnUyZlJLWXA0ZVHSAaoBQVVfeXFMT3BwVV9lZzBQRTFjWUNVNEFzaUlhOUJuTHByVVRhdjRTbjdpajdOTjRtc2hfOEotMWlSb0FvX1F3azI2czNjMHREWnRJbFptM0F5ZHJkWUFsMW5fMDBsNU1YODgzT2VkMWZacU51MzkxaHJ0S216TF9UR241SnM0OVo2eHlDM0F6V2VfbUt4elZfZVBub2pLNW5fazhqV1hNUnBzRmkxS0NUQVE?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMingFBVV95cUxOYzFrN28yN3RDREhxYV9CVHl3UGU1NlpvSFJqaHJGWVpraVhEOEtqTnZVQk1OTjVjX1djWENocHdtYy1WY1dBSHZncjg3aGxWOXlwcFktaVVxYzBmZllLbzBaLUUxSEpyNW1HX3V5MG9YMWhTcjNfcnZxQ1JKRHZkMjlYSjlmUHk1SGFEYy0tYmlqWE96ajBqUnNSS19TUQ?oc=5</t>
         </is>
       </c>
       <c r="I45" s="2" t="inlineStr"/>
@@ -2496,12 +2496,12 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>Corporate Tax</t>
+          <t>VAT</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
@@ -2511,7 +2511,7 @@
       </c>
       <c r="E46" s="3" t="inlineStr">
         <is>
-          <t>UAE extends Corporate Tax relief until 2029 for businesses earning up to $817,000 - Arabian Business</t>
+          <t>UAE seizes 3.58 million non-compliant excise goods - Gulf News</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
@@ -2526,7 +2526,7 @@
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMieEFVX3lxTE5SM3FoRTVUSmJwTlpLbi1vOGFPM3RPcXpraXlCUG9iQlhuUUJ2MGRCczd6aDM0MFFNWS0yS2tNNVIxYjd2Y3AxWExhUnJNcHNXT3dLdGhyV2FBQUQwbmZ3YjRZc3NXTkNoLU5HTFRkTWRkSlZ6TEtHbg?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMipwFBVV95cUxOOF9vUDk3UXlsY19FUWtOOEJ2V3Awam9fY09zeS1seXpTUUt2Y05TQlVUVjlwYlVuX2hRN3JBM095eTlqZ3pxWWx5ZWJzUzV1bGdCQ21JMzd1bjRIMGRMdHpiZWVOM1lmOVdtSXlicW4wYUNoYjMySjFTNl9OTnRvYWZycGdhODlTcU9sQUpwUEdJcnltNF9nSXpBWkpJbjF0VG1qeVJqTdIBugFBVV95cUxPMDVISGFVMTVqWFFiS0VMTmlzZzlyWXRVUl9BTjBGaWgtS21lN05BdlppYlVNQkNtYmZWaHRIczNlSWRmbXBBdG9zamlobjFhTFh6R2lYZFJ1RUtKWGZqOWpNd21LTmNxaUF1SjVIUm9UNjF6cmwxUGY2ZHFIVHBFdVJNMXcyeFp3dUZ2V1hpVmtnRmZOY29nLWNWQmxsQ0tHUzd0RjRyRUlZeW1adThtZEpPVl9KT1pFRUE?oc=5</t>
         </is>
       </c>
       <c r="I46" s="2" t="inlineStr"/>
@@ -2556,7 +2556,7 @@
       </c>
       <c r="E47" s="3" t="inlineStr">
         <is>
-          <t>Ministry of Finance announces extension of small business relief for corporate tax purposes until 31 December 2029 - Zawya</t>
+          <t>UAE Extends Small Business Relief for Corporate Tax to 2029 - tbreak.com</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
@@ -2571,7 +2571,7 @@
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMihwJBVV95cUxOWVAwdTI2R09XSWRHaFNWYkNGdUJsSTNnaGpRandNeklubW8zM2h3VkNIcmRiQTVrZUxlSnhydWtqUGVTRS1vYVVQWWJfY2swUzhYOFJrdHVCQTlvTk1LNVBfWjBPbHZxWVU5Q0xQVWFHbTlLYlE0ek1aWFhqaUF3dDlTY2p2T0dtV3gzSXhaWkdFdWFBejA5ZkhDSkVPanZUWDk0d1oxNlJOUkNxMER2M1oyc3Nla2NnUW9WYmFRS04zeGlCcjQ1YVNZT2ZraU5EN0h2ZWRDaklZTjFQUklLWmRGRVFkUjhKUjBybHA5UktLZHFiVnUtOFpuNmhSZ0o3YVV3eld3WQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMifEFVX3lxTE9icS1QSXhYc09ROHVJdzRtdXJTMEdLa0o5Mm5TZ3VxR002a3lTeFR5anZqRmNtcVEyQWxfQ050UFVOZnFBcFdwT1VoNGlVZU9xYkY2WkM5SlpSSnp6QkpHck5rTUxqOXNjNjM0UmFTQkFfOXZySFFON1pCSXc?oc=5</t>
         </is>
       </c>
       <c r="I47" s="2" t="inlineStr"/>
@@ -2586,7 +2586,7 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
@@ -2601,7 +2601,7 @@
       </c>
       <c r="E48" s="3" t="inlineStr">
         <is>
-          <t>FTA reminds small businesses to file corporate tax returns - Sharjah24</t>
+          <t>UAE extends corporate tax relief for small businesses until end of 2029 - Gulf News</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
@@ -2616,7 +2616,7 @@
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiW0FVX3lxTE5NZ1VTdFlkVERkd0pETmFiVUQzZzEySVNaeWFyV2N3MHdhSWZreEZnUDFCYXhiWGtCOVVxMFdWUzhDa3JCU1czenE3QzJzaG0tNU5iMkFmRFRsTUU?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMixgFBVV95cUxNNEo4Tm9qN1dERmwzZ0tMR0ZOSUVQTkpOTTNiTDc1U2VaSTkyRkExekRzRjUzb2xrelYzV0oydU1qS2JCbHJXd1hxeWhPdmtUN1UtcXRCOHZpSXBxMlBMdFRKbDNxYlNFaVdwRXROTUVxWC1tZUpObDVIZzNVUDEzSUZpNkIxN3ctTDRNWU9xOUx6QXZieFdVV1hkNHhlcldHUzY5b21BZ1J2VTVhMlN2a1V5V1dJRkw1OTItdWo5Qzk5N2lPX1HSAdgBQVVfeXFMTmRQM08wYWhkelVySDhudHZWLWQyZ2lyUG9TNEJhWVV6ejAybDV6QXdvUFR5ZndxZldxWHVDMjRKVm1Ndm0yeE1HZHo1LXoyVFBzMkhuUDZESEw5RUFIaWlfNEdObjNxRlc4VFpOZVQ3RDhhellsdEpYN3pLVzl1d1Fva3R0RWpDb0d5cVN0Z3I3emowS2tNbkplWTh1Z2NvVkRMd0R3STNWV3hrUVFtd3hxdjQxWjI2ZU4wVE9JTzlsWVUwYXlPTmU4YWJmazMxQk93MHVHbGZE?oc=5</t>
         </is>
       </c>
       <c r="I48" s="2" t="inlineStr"/>
@@ -2631,7 +2631,7 @@
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
@@ -2646,7 +2646,7 @@
       </c>
       <c r="E49" s="3" t="inlineStr">
         <is>
-          <t>UAE extends small business relief for corporate tax until December 2029 - TradeArabia</t>
+          <t>Small businesses in UAE urged to file corporate tax returns before deadline, says FTA - khaleejtimes.com</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
@@ -2661,7 +2661,7 @@
       </c>
       <c r="H49" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxOc3RJWW11LUNyUERIeHh0dTVRVFJySzBoWVB0N1RCdVNpTVpORW03RkVXaG1pdk5HbWJfTDUzYXRIellIdlo4dVBXcXpuZHNrQXZRMk5MMGF1UkpqbGRTbXZRekZTYkU3cHpsdmJHdTVRdFFxSE1aSzZxWW1rb0RuT1RNZzVOWG91OGVTcFZVUGFVLWRUY3JsRnEtYkR4WUJjWnp6NkljSUd2NExsdUYtVA?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxOWnJlYmRmRm4xdy0xZ0toMUNUbnhTd3A5UW1pVzhFeXhIM2txamo4NU5qYVYwZGlQcEYwLTJhelBkOEdHajRYSE5PRnZtdmxGWmc0R2JlUVk0eVc0aW53NzdlM08zeWFzTUNocU9UcnY3UTNhTHVzZHhjRXFPZ0ZMMHMyRExEcjFiVVhKVzMxYk9FSHUxdERQRnUyZlJLWXA0ZVHSAaoBQVVfeXFMT3BwVV9lZzBQRTFjWUNVNEFzaUlhOUJuTHByVVRhdjRTbjdpajdOTjRtc2hfOEotMWlSb0FvX1F3azI2czNjMHREWnRJbFptM0F5ZHJkWUFsMW5fMDBsNU1YODgzT2VkMWZacU51MzkxaHJ0S216TF9UR241SnM0OVo2eHlDM0F6V2VfbUt4elZfZVBub2pLNW5fazhqV1hNUnBzRmkxS0NUQVE?oc=5</t>
         </is>
       </c>
       <c r="I49" s="2" t="inlineStr"/>
@@ -2676,7 +2676,7 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
@@ -2691,7 +2691,7 @@
       </c>
       <c r="E50" s="3" t="inlineStr">
         <is>
-          <t>UAE tax warning as thousands of businesses approach Corporate Tax deadline - Arabian Business</t>
+          <t>UAE extends Corporate Tax relief until 2029 for businesses earning up to $817,000 - Arabian Business</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
@@ -2706,7 +2706,7 @@
       </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMidEFVX3lxTFBGbVZOWkkxM2FaVGlfeENJVWJXYzN6SDdmNk9nOFBYWWJDV3N6eGxVcnBRRXc5cDY5Qy1xSnNBQzVHMXR3NGpacEVucjlTMFRSaHc0dG5aZXc1aUVwSXlrTXhFTGd3RWNMbzVpWmdEVUZuUC1N?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMieEFVX3lxTE5SM3FoRTVUSmJwTlpLbi1vOGFPM3RPcXpraXlCUG9iQlhuUUJ2MGRCczd6aDM0MFFNWS0yS2tNNVIxYjd2Y3AxWExhUnJNcHNXT3dLdGhyV2FBQUQwbmZ3YjRZc3NXTkNoLU5HTFRkTWRkSlZ6TEtHbg?oc=5</t>
         </is>
       </c>
       <c r="I50" s="2" t="inlineStr"/>
@@ -2721,7 +2721,7 @@
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
@@ -2736,7 +2736,7 @@
       </c>
       <c r="E51" s="3" t="inlineStr">
         <is>
-          <t>UAE reminds small businesses to file corporate tax returns even if no tax is due - Gulf News</t>
+          <t>Ministry of Finance announces extension of small business relief for corporate tax purposes until 31 December 2029 - Zawya</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
@@ -2751,7 +2751,7 @@
       </c>
       <c r="H51" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMi0gFBVV95cUxOTm96UlB4Q2xPRlcybWNBanAtYXhxQkg0eHVCNDBvZlZGTWNGNzlSekNuVWZCU1JvOWR4MWxLanJMZEsyRms3NnZDSU90RnZuTkhad3pLLU1XX2VWV215T21HMTBmbVF1X0hmakhwM1BYZVNUQXZEV3A1UmR0QkZxVlJ1VDV5dGVMMFJFSGRxckpYVkVMMmFNMFBBdE9MZnlFSjJ3MDFXNzg2UXd0SUthQlZrd1Zjdy1JTVFkMEZlU0VKc3lzQW84VDBGLXFfVF93SnfSAeQBQVVfeXFMUEpicHFURTEyaDByTG44RGZUZ2R0MGJwRmdpV0hydzNTdkVYd0lFZzNITm9ueldCQ0JUZjZ3dW1TZ0xCSHM1S3c5eXExQlZac3V6bGd5Q1EzWFljOVRrZkJWRV9XcnFQWHdzRHQzWDRiUFhHaXlKMldlZHp5YW9zMHh2emxiX0R3MXdva2NFZ2JwcnVBZk52dEh2UEhvTW9FYzlJQ2xWdWZPQmpteFpaWnNUV0lpUTRiT0hNRXdHQVg1Q1VibWZqVWdocjBVVHJtVVFUbVFBdjJoRndFUS1aMTc5SEVh?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMihwJBVV95cUxOWVAwdTI2R09XSWRHaFNWYkNGdUJsSTNnaGpRandNeklubW8zM2h3VkNIcmRiQTVrZUxlSnhydWtqUGVTRS1vYVVQWWJfY2swUzhYOFJrdHVCQTlvTk1LNVBfWjBPbHZxWVU5Q0xQVWFHbTlLYlE0ek1aWFhqaUF3dDlTY2p2T0dtV3gzSXhaWkdFdWFBejA5ZkhDSkVPanZUWDk0d1oxNlJOUkNxMER2M1oyc3Nla2NnUW9WYmFRS04zeGlCcjQ1YVNZT2ZraU5EN0h2ZWRDaklZTjFQUklLWmRGRVFkUjhKUjBybHA5UktLZHFiVnUtOFpuNmhSZ0o3YVV3eld3WQ?oc=5</t>
         </is>
       </c>
       <c r="I51" s="2" t="inlineStr"/>
@@ -2771,7 +2771,7 @@
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>VAT</t>
+          <t>Corporate Tax</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
@@ -2781,7 +2781,7 @@
       </c>
       <c r="E52" s="3" t="inlineStr">
         <is>
-          <t>Federal Tax Authority wins SAP Global Innovation Award - SAP News Center</t>
+          <t>FTA reminds small businesses to file corporate tax returns - Sharjah24</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
@@ -2796,7 +2796,7 @@
       </c>
       <c r="H52" s="2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxQYWE1ODFVeGZ2UEVVd0IyYXY0ckdPdFp4blEzcm9pZTZ5dm1MUDlocTNzNnd4dTh3cVhQb0o2aHJ2Y2VjTndrd2d6N2t1eW9OTzVtQ2JrcXVwN2NidFd2WUViQlRleTVQQXNpV2VvOVkyMFRINHhnNXpsUWdOcDhDUk1TbkpTajRkcUFGblBfWXhRZVU?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiW0FVX3lxTE5NZ1VTdFlkVERkd0pETmFiVUQzZzEySVNaeWFyV2N3MHdhSWZreEZnUDFCYXhiWGtCOVVxMFdWUzhDa3JCU1czenE3QzJzaG0tNU5iMkFmRFRsTUU?oc=5</t>
         </is>
       </c>
       <c r="I52" s="2" t="inlineStr"/>
@@ -2809,35 +2809,39 @@
           <t>2026-08-09</t>
         </is>
       </c>
-      <c r="B53" s="2" t="inlineStr"/>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Corporate Tax</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>official</t>
+          <t>news</t>
         </is>
       </c>
       <c r="E53" s="3" t="inlineStr">
         <is>
-          <t>Ministry of Finance Adopts “Aani” and “Jaywan” as New Payment Channels for Federal Service Fees and Fines</t>
+          <t>UAE extends small business relief for corporate tax until December 2029 - TradeArabia</t>
         </is>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>Ministry of Finance — News</t>
+          <t>News — UAE Corporate Tax</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t>mof.gov.ae</t>
+          <t>news.google.com</t>
         </is>
       </c>
       <c r="H53" s="2" t="inlineStr">
         <is>
-          <t>https://mof.gov.ae/en/news/ministry-of-finance-adopts-aani-and-jaywan-as-new-payment-channels-for-federal-service-fees-and-fines/</t>
+          <t>https://news.google.com/rss/articles/CBMisAFBVV95cUxOc3RJWW11LUNyUERIeHh0dTVRVFJySzBoWVB0N1RCdVNpTVpORW03RkVXaG1pdk5HbWJfTDUzYXRIellIdlo4dVBXcXpuZHNrQXZRMk5MMGF1UkpqbGRTbXZRekZTYkU3cHpsdmJHdTVRdFFxSE1aSzZxWW1rb0RuT1RNZzVOWG91OGVTcFZVUGFVLWRUY3JsRnEtYkR4WUJjWnp6NkljSUd2NExsdUYtVA?oc=5</t>
         </is>
       </c>
       <c r="I53" s="2" t="inlineStr"/>
@@ -2850,35 +2854,39 @@
           <t>2026-08-09</t>
         </is>
       </c>
-      <c r="B54" s="2" t="inlineStr"/>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>VAT</t>
+          <t>Corporate Tax</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>official</t>
+          <t>news</t>
         </is>
       </c>
       <c r="E54" s="3" t="inlineStr">
         <is>
-          <t>Ministry of Finance Announces Decision introduces a Minimum Excise Price for Liquids Used in Electronic Smoking Devices Effective 1 September 2026</t>
+          <t>UAE tax warning as thousands of businesses approach Corporate Tax deadline - Arabian Business</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>Ministry of Finance — News</t>
+          <t>News — UAE Corporate Tax</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>mof.gov.ae</t>
+          <t>news.google.com</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr">
         <is>
-          <t>https://mof.gov.ae/en/news/ministry-of-finance-announces-decision-introduces-a-minimum-excise-price-for-liquids-used-in-electronic-smoking-devices-effective-1-september-2026/</t>
+          <t>https://news.google.com/rss/articles/CBMidEFVX3lxTFBGbVZOWkkxM2FaVGlfeENJVWJXYzN6SDdmNk9nOFBYWWJDV3N6eGxVcnBRRXc5cDY5Qy1xSnNBQzVHMXR3NGpacEVucjlTMFRSaHc0dG5aZXc1aUVwSXlrTXhFTGd3RWNMbzVpWmdEVUZuUC1N?oc=5</t>
         </is>
       </c>
       <c r="I54" s="2" t="inlineStr"/>
@@ -2891,7 +2899,11 @@
           <t>2026-08-09</t>
         </is>
       </c>
-      <c r="B55" s="2" t="inlineStr"/>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
           <t>Corporate Tax</t>
@@ -2899,32 +2911,200 @@
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>official</t>
+          <t>news</t>
         </is>
       </c>
       <c r="E55" s="3" t="inlineStr">
         <is>
-          <t>Ministry of Finance Announces Extension of Small Business Relief for Corporate Tax Purposes until 31 December 2029</t>
+          <t>UAE reminds small businesses to file corporate tax returns even if no tax is due - Gulf News</t>
         </is>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>Ministry of Finance — News</t>
+          <t>News — UAE Corporate Tax</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>mof.gov.ae</t>
+          <t>news.google.com</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr">
         <is>
-          <t>https://mof.gov.ae/en/news/ministry-of-finance-announces-extension-of-small-business-relief-for-corporate-tax-purposes-until-31-december-2029/</t>
+          <t>https://news.google.com/rss/articles/CBMi0gFBVV95cUxOTm96UlB4Q2xPRlcybWNBanAtYXhxQkg0eHVCNDBvZlZGTWNGNzlSekNuVWZCU1JvOWR4MWxLanJMZEsyRms3NnZDSU90RnZuTkhad3pLLU1XX2VWV215T21HMTBmbVF1X0hmakhwM1BYZVNUQXZEV3A1UmR0QkZxVlJ1VDV5dGVMMFJFSGRxckpYVkVMMmFNMFBBdE9MZnlFSjJ3MDFXNzg2UXd0SUthQlZrd1Zjdy1JTVFkMEZlU0VKc3lzQW84VDBGLXFfVF93SnfSAeQBQVVfeXFMUEpicHFURTEyaDByTG44RGZUZ2R0MGJwRmdpV0hydzNTdkVYd0lFZzNITm9ueldCQ0JUZjZ3dW1TZ0xCSHM1S3c5eXExQlZac3V6bGd5Q1EzWFljOVRrZkJWRV9XcnFQWHdzRHQzWDRiUFhHaXlKMldlZHp5YW9zMHh2emxiX0R3MXdva2NFZ2JwcnVBZk52dEh2UEhvTW9FYzlJQ2xWdWZPQmpteFpaWnNUV0lpUTRiT0hNRXdHQVg1Q1VibWZqVWdocjBVVHJtVVFUbVFBdjJoRndFUS1aMTc5SEVh?oc=5</t>
         </is>
       </c>
       <c r="I55" s="2" t="inlineStr"/>
       <c r="J55" s="2" t="inlineStr"/>
       <c r="K55" s="2" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>VAT</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>news</t>
+        </is>
+      </c>
+      <c r="E56" s="3" t="inlineStr">
+        <is>
+          <t>Federal Tax Authority wins SAP Global Innovation Award - SAP News Center</t>
+        </is>
+      </c>
+      <c r="F56" s="2" t="inlineStr">
+        <is>
+          <t>News — UAE Corporate Tax</t>
+        </is>
+      </c>
+      <c r="G56" s="2" t="inlineStr">
+        <is>
+          <t>news.google.com</t>
+        </is>
+      </c>
+      <c r="H56" s="2" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMikwFBVV95cUxQYWE1ODFVeGZ2UEVVd0IyYXY0ckdPdFp4blEzcm9pZTZ5dm1MUDlocTNzNnd4dTh3cVhQb0o2aHJ2Y2VjTndrd2d6N2t1eW9OTzVtQ2JrcXVwN2NidFd2WUViQlRleTVQQXNpV2VvOVkyMFRINHhnNXpsUWdOcDhDUk1TbkpTajRkcUFGblBfWXhRZVU?oc=5</t>
+        </is>
+      </c>
+      <c r="I56" s="2" t="inlineStr"/>
+      <c r="J56" s="2" t="inlineStr"/>
+      <c r="K56" s="2" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr"/>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>official</t>
+        </is>
+      </c>
+      <c r="E57" s="3" t="inlineStr">
+        <is>
+          <t>Ministry of Finance Adopts “Aani” and “Jaywan” as New Payment Channels for Federal Service Fees and Fines</t>
+        </is>
+      </c>
+      <c r="F57" s="2" t="inlineStr">
+        <is>
+          <t>Ministry of Finance — News</t>
+        </is>
+      </c>
+      <c r="G57" s="2" t="inlineStr">
+        <is>
+          <t>mof.gov.ae</t>
+        </is>
+      </c>
+      <c r="H57" s="2" t="inlineStr">
+        <is>
+          <t>https://mof.gov.ae/en/news/ministry-of-finance-adopts-aani-and-jaywan-as-new-payment-channels-for-federal-service-fees-and-fines/</t>
+        </is>
+      </c>
+      <c r="I57" s="2" t="inlineStr"/>
+      <c r="J57" s="2" t="inlineStr"/>
+      <c r="K57" s="2" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr"/>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>VAT</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>official</t>
+        </is>
+      </c>
+      <c r="E58" s="3" t="inlineStr">
+        <is>
+          <t>Ministry of Finance Announces Decision introduces a Minimum Excise Price for Liquids Used in Electronic Smoking Devices Effective 1 September 2026</t>
+        </is>
+      </c>
+      <c r="F58" s="2" t="inlineStr">
+        <is>
+          <t>Ministry of Finance — News</t>
+        </is>
+      </c>
+      <c r="G58" s="2" t="inlineStr">
+        <is>
+          <t>mof.gov.ae</t>
+        </is>
+      </c>
+      <c r="H58" s="2" t="inlineStr">
+        <is>
+          <t>https://mof.gov.ae/en/news/ministry-of-finance-announces-decision-introduces-a-minimum-excise-price-for-liquids-used-in-electronic-smoking-devices-effective-1-september-2026/</t>
+        </is>
+      </c>
+      <c r="I58" s="2" t="inlineStr"/>
+      <c r="J58" s="2" t="inlineStr"/>
+      <c r="K58" s="2" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr"/>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>Corporate Tax</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="inlineStr">
+        <is>
+          <t>official</t>
+        </is>
+      </c>
+      <c r="E59" s="3" t="inlineStr">
+        <is>
+          <t>Ministry of Finance Announces Extension of Small Business Relief for Corporate Tax Purposes until 31 December 2029</t>
+        </is>
+      </c>
+      <c r="F59" s="2" t="inlineStr">
+        <is>
+          <t>Ministry of Finance — News</t>
+        </is>
+      </c>
+      <c r="G59" s="2" t="inlineStr">
+        <is>
+          <t>mof.gov.ae</t>
+        </is>
+      </c>
+      <c r="H59" s="2" t="inlineStr">
+        <is>
+          <t>https://mof.gov.ae/en/news/ministry-of-finance-announces-extension-of-small-business-relief-for-corporate-tax-purposes-until-31-december-2029/</t>
+        </is>
+      </c>
+      <c r="I59" s="2" t="inlineStr"/>
+      <c r="J59" s="2" t="inlineStr"/>
+      <c r="K59" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>